<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@40f2974c5ad5a300fd0063addb753dd64f14e2ce 🚀
</commit_message>
<xml_diff>
--- a/StructureDefinition-Procedure.xlsx
+++ b/StructureDefinition-Procedure.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-01-06T16:52:49+00:00</t>
+    <t>2025-01-06T17:00:55+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -11161,7 +11161,7 @@
         <v>96</v>
       </c>
       <c r="H64" t="s" s="2">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="I64" t="s" s="2">
         <v>88</v>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@7d9bfd1c890c74d12f9540b5f6f5f29049bd3ba6 🚀
</commit_message>
<xml_diff>
--- a/StructureDefinition-Procedure.xlsx
+++ b/StructureDefinition-Procedure.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4340" uniqueCount="601">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4339" uniqueCount="602">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-02-24T16:22:43+00:00</t>
+    <t>2025-02-25T09:38:10+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -890,6 +890,9 @@
   </si>
   <si>
     <t>Allows for translations and alternate encodings within a code system.  Also supports communication of the same instance to systems requiring different encodings.</t>
+  </si>
+  <si>
+    <t>http://fhir.hl7.nl/zorgviewer/ValueSet/VerrichtingTypeCodelist</t>
   </si>
   <si>
     <t xml:space="preserve">value:system}
@@ -6091,7 +6094,7 @@
         <v>87</v>
       </c>
       <c r="H28" t="s" s="2">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="I28" t="s" s="2">
         <v>88</v>
@@ -6137,19 +6140,17 @@
         <v>88</v>
       </c>
       <c r="X28" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="Y28" t="s" s="2">
-        <v>88</v>
-      </c>
+        <v>119</v>
+      </c>
+      <c r="Y28" s="2"/>
       <c r="Z28" t="s" s="2">
-        <v>88</v>
+        <v>277</v>
       </c>
       <c r="AA28" t="s" s="2">
         <v>88</v>
       </c>
       <c r="AB28" t="s" s="2">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="AC28" s="2"/>
       <c r="AD28" t="s" s="2">
@@ -6159,7 +6160,7 @@
         <v>145</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>86</v>
@@ -6204,27 +6205,27 @@
         <v>88</v>
       </c>
       <c r="AU28" t="s" s="2">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="AV28" t="s" s="2">
         <v>88</v>
       </c>
       <c r="AW28" t="s" s="2">
-        <v>280</v>
+        <v>281</v>
       </c>
     </row>
     <row r="29" hidden="true">
       <c r="A29" t="s" s="2">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B29" t="s" s="2">
         <v>271</v>
       </c>
       <c r="C29" t="s" s="2">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D29" t="s" s="2">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="E29" s="2"/>
       <c r="F29" t="s" s="2">
@@ -6249,7 +6250,7 @@
         <v>260</v>
       </c>
       <c r="M29" t="s" s="2">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="N29" t="s" s="2">
         <v>275</v>
@@ -6283,10 +6284,10 @@
         <v>231</v>
       </c>
       <c r="Y29" t="s" s="2">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="Z29" t="s" s="2">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="AA29" t="s" s="2">
         <v>88</v>
@@ -6304,7 +6305,7 @@
         <v>88</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="AG29" t="s" s="2">
         <v>86</v>
@@ -6349,21 +6350,21 @@
         <v>88</v>
       </c>
       <c r="AU29" t="s" s="2">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="AV29" t="s" s="2">
         <v>88</v>
       </c>
       <c r="AW29" t="s" s="2">
-        <v>280</v>
+        <v>281</v>
       </c>
     </row>
     <row r="30" hidden="true">
       <c r="A30" t="s" s="2">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
@@ -6499,10 +6500,10 @@
     </row>
     <row r="31" hidden="true">
       <c r="A31" t="s" s="2">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
@@ -6640,10 +6641,10 @@
     </row>
     <row r="32" hidden="true">
       <c r="A32" t="s" s="2">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
@@ -6669,23 +6670,23 @@
         <v>109</v>
       </c>
       <c r="L32" t="s" s="2">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="M32" t="s" s="2">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="N32" t="s" s="2">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="O32" t="s" s="2">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="P32" t="s" s="2">
         <v>88</v>
       </c>
       <c r="Q32" s="2"/>
       <c r="R32" t="s" s="2">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="S32" t="s" s="2">
         <v>88</v>
@@ -6727,7 +6728,7 @@
         <v>88</v>
       </c>
       <c r="AF32" t="s" s="2">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>86</v>
@@ -6772,21 +6773,21 @@
         <v>88</v>
       </c>
       <c r="AU32" t="s" s="2">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="AV32" t="s" s="2">
         <v>88</v>
       </c>
       <c r="AW32" t="s" s="2">
-        <v>300</v>
+        <v>301</v>
       </c>
     </row>
     <row r="33" hidden="true">
       <c r="A33" t="s" s="2">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
@@ -6812,13 +6813,13 @@
         <v>157</v>
       </c>
       <c r="L33" t="s" s="2">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="M33" t="s" s="2">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="N33" t="s" s="2">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="O33" s="2"/>
       <c r="P33" t="s" s="2">
@@ -6868,7 +6869,7 @@
         <v>88</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="AG33" t="s" s="2">
         <v>86</v>
@@ -6913,21 +6914,21 @@
         <v>88</v>
       </c>
       <c r="AU33" t="s" s="2">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="AV33" t="s" s="2">
         <v>88</v>
       </c>
       <c r="AW33" t="s" s="2">
-        <v>308</v>
+        <v>309</v>
       </c>
     </row>
     <row r="34" hidden="true">
       <c r="A34" t="s" s="2">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
@@ -6953,14 +6954,14 @@
         <v>115</v>
       </c>
       <c r="L34" t="s" s="2">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="M34" t="s" s="2">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="N34" s="2"/>
       <c r="O34" t="s" s="2">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="P34" t="s" s="2">
         <v>88</v>
@@ -7009,7 +7010,7 @@
         <v>88</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="AG34" t="s" s="2">
         <v>86</v>
@@ -7054,21 +7055,21 @@
         <v>88</v>
       </c>
       <c r="AU34" t="s" s="2">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="AV34" t="s" s="2">
         <v>88</v>
       </c>
       <c r="AW34" t="s" s="2">
-        <v>316</v>
+        <v>317</v>
       </c>
     </row>
     <row r="35" hidden="true">
       <c r="A35" t="s" s="2">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
@@ -7094,14 +7095,14 @@
         <v>157</v>
       </c>
       <c r="L35" t="s" s="2">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="M35" t="s" s="2">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="N35" s="2"/>
       <c r="O35" t="s" s="2">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="P35" t="s" s="2">
         <v>88</v>
@@ -7150,7 +7151,7 @@
         <v>88</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="AG35" t="s" s="2">
         <v>86</v>
@@ -7195,21 +7196,21 @@
         <v>88</v>
       </c>
       <c r="AU35" t="s" s="2">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="AV35" t="s" s="2">
         <v>88</v>
       </c>
       <c r="AW35" t="s" s="2">
-        <v>324</v>
+        <v>325</v>
       </c>
     </row>
     <row r="36" hidden="true">
       <c r="A36" t="s" s="2">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
@@ -7235,16 +7236,16 @@
         <v>237</v>
       </c>
       <c r="L36" t="s" s="2">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="M36" t="s" s="2">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="N36" t="s" s="2">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="O36" t="s" s="2">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="P36" t="s" s="2">
         <v>88</v>
@@ -7293,7 +7294,7 @@
         <v>88</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>86</v>
@@ -7338,21 +7339,21 @@
         <v>88</v>
       </c>
       <c r="AU36" t="s" s="2">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="AV36" t="s" s="2">
         <v>88</v>
       </c>
       <c r="AW36" t="s" s="2">
-        <v>333</v>
+        <v>334</v>
       </c>
     </row>
     <row r="37" hidden="true">
       <c r="A37" t="s" s="2">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
@@ -7378,16 +7379,16 @@
         <v>157</v>
       </c>
       <c r="L37" t="s" s="2">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="M37" t="s" s="2">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="N37" t="s" s="2">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="O37" t="s" s="2">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="P37" t="s" s="2">
         <v>88</v>
@@ -7436,7 +7437,7 @@
         <v>88</v>
       </c>
       <c r="AF37" t="s" s="2">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="AG37" t="s" s="2">
         <v>86</v>
@@ -7481,25 +7482,25 @@
         <v>88</v>
       </c>
       <c r="AU37" t="s" s="2">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="AV37" t="s" s="2">
         <v>88</v>
       </c>
       <c r="AW37" t="s" s="2">
-        <v>341</v>
+        <v>342</v>
       </c>
     </row>
     <row r="38" hidden="true">
       <c r="A38" t="s" s="2">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="E38" s="2"/>
       <c r="F38" t="s" s="2">
@@ -7518,13 +7519,13 @@
         <v>97</v>
       </c>
       <c r="K38" t="s" s="2">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="L38" t="s" s="2">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="M38" t="s" s="2">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="N38" s="2"/>
       <c r="O38" s="2"/>
@@ -7575,7 +7576,7 @@
         <v>88</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>96</v>
@@ -7599,7 +7600,7 @@
         <v>88</v>
       </c>
       <c r="AN38" t="s" s="2">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="AO38" t="s" s="2">
         <v>88</v>
@@ -7620,25 +7621,25 @@
         <v>88</v>
       </c>
       <c r="AU38" t="s" s="2">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="AV38" t="s" s="2">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="AW38" t="s" s="2">
-        <v>350</v>
+        <v>351</v>
       </c>
     </row>
     <row r="39" hidden="true">
       <c r="A39" t="s" s="2">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="E39" s="2"/>
       <c r="F39" t="s" s="2">
@@ -7657,13 +7658,13 @@
         <v>97</v>
       </c>
       <c r="K39" t="s" s="2">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="L39" t="s" s="2">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="M39" t="s" s="2">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="N39" s="2"/>
       <c r="O39" s="2"/>
@@ -7714,7 +7715,7 @@
         <v>88</v>
       </c>
       <c r="AF39" t="s" s="2">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="AG39" t="s" s="2">
         <v>86</v>
@@ -7759,21 +7760,21 @@
         <v>88</v>
       </c>
       <c r="AU39" t="s" s="2">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="AV39" t="s" s="2">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="AW39" t="s" s="2">
-        <v>358</v>
+        <v>359</v>
       </c>
     </row>
     <row r="40" hidden="true">
       <c r="A40" t="s" s="2">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
@@ -7796,13 +7797,13 @@
         <v>97</v>
       </c>
       <c r="K40" t="s" s="2">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="L40" t="s" s="2">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="M40" t="s" s="2">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="N40" s="2"/>
       <c r="O40" s="2"/>
@@ -7841,17 +7842,17 @@
         <v>88</v>
       </c>
       <c r="AB40" t="s" s="2">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="AC40" s="2"/>
       <c r="AD40" t="s" s="2">
         <v>88</v>
       </c>
       <c r="AE40" t="s" s="2">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="AF40" t="s" s="2">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="AG40" t="s" s="2">
         <v>86</v>
@@ -7875,7 +7876,7 @@
         <v>88</v>
       </c>
       <c r="AN40" t="s" s="2">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="AO40" t="s" s="2">
         <v>88</v>
@@ -7896,24 +7897,24 @@
         <v>88</v>
       </c>
       <c r="AU40" t="s" s="2">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="AV40" t="s" s="2">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="AW40" t="s" s="2">
-        <v>368</v>
+        <v>369</v>
       </c>
     </row>
     <row r="41" hidden="true">
       <c r="A41" t="s" s="2">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="C41" t="s" s="2">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="D41" t="s" s="2">
         <v>88</v>
@@ -7935,13 +7936,13 @@
         <v>97</v>
       </c>
       <c r="K41" t="s" s="2">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="L41" t="s" s="2">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="M41" t="s" s="2">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="N41" s="2"/>
       <c r="O41" s="2"/>
@@ -7992,7 +7993,7 @@
         <v>88</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="AG41" t="s" s="2">
         <v>86</v>
@@ -8037,21 +8038,21 @@
         <v>88</v>
       </c>
       <c r="AU41" t="s" s="2">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="AV41" t="s" s="2">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="AW41" t="s" s="2">
-        <v>368</v>
+        <v>369</v>
       </c>
     </row>
     <row r="42" hidden="true">
       <c r="A42" t="s" s="2">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
@@ -8187,10 +8188,10 @@
     </row>
     <row r="43" hidden="true">
       <c r="A43" t="s" s="2">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
@@ -8328,14 +8329,14 @@
     </row>
     <row r="44" hidden="true">
       <c r="A44" t="s" s="2">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="E44" s="2"/>
       <c r="F44" t="s" s="2">
@@ -8354,16 +8355,16 @@
         <v>97</v>
       </c>
       <c r="K44" t="s" s="2">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="L44" t="s" s="2">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="M44" t="s" s="2">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="N44" t="s" s="2">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="O44" s="2"/>
       <c r="P44" t="s" s="2">
@@ -8413,7 +8414,7 @@
         <v>88</v>
       </c>
       <c r="AF44" t="s" s="2">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="AG44" t="s" s="2">
         <v>86</v>
@@ -8422,13 +8423,13 @@
         <v>96</v>
       </c>
       <c r="AI44" t="s" s="2">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="AJ44" t="s" s="2">
         <v>88</v>
       </c>
       <c r="AK44" t="s" s="2">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="AL44" t="s" s="2">
         <v>88</v>
@@ -8440,7 +8441,7 @@
         <v>88</v>
       </c>
       <c r="AO44" t="s" s="2">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="AP44" t="s" s="2">
         <v>88</v>
@@ -8449,7 +8450,7 @@
         <v>88</v>
       </c>
       <c r="AR44" t="s" s="2">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="AS44" t="s" s="2">
         <v>88</v>
@@ -8458,25 +8459,25 @@
         <v>88</v>
       </c>
       <c r="AU44" t="s" s="2">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="AV44" t="s" s="2">
         <v>88</v>
       </c>
       <c r="AW44" t="s" s="2">
-        <v>386</v>
+        <v>387</v>
       </c>
     </row>
     <row r="45" hidden="true">
       <c r="A45" t="s" s="2">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="E45" s="2"/>
       <c r="F45" t="s" s="2">
@@ -8495,23 +8496,23 @@
         <v>97</v>
       </c>
       <c r="K45" t="s" s="2">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="L45" t="s" s="2">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="M45" t="s" s="2">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="N45" t="s" s="2">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="O45" s="2"/>
       <c r="P45" t="s" s="2">
         <v>88</v>
       </c>
       <c r="Q45" t="s" s="2">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="R45" t="s" s="2">
         <v>88</v>
@@ -8556,7 +8557,7 @@
         <v>88</v>
       </c>
       <c r="AF45" t="s" s="2">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="AG45" t="s" s="2">
         <v>86</v>
@@ -8565,13 +8566,13 @@
         <v>96</v>
       </c>
       <c r="AI45" t="s" s="2">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="AJ45" t="s" s="2">
         <v>88</v>
       </c>
       <c r="AK45" t="s" s="2">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="AL45" t="s" s="2">
         <v>88</v>
@@ -8583,7 +8584,7 @@
         <v>88</v>
       </c>
       <c r="AO45" t="s" s="2">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="AP45" t="s" s="2">
         <v>88</v>
@@ -8592,7 +8593,7 @@
         <v>88</v>
       </c>
       <c r="AR45" t="s" s="2">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="AS45" t="s" s="2">
         <v>88</v>
@@ -8601,25 +8602,25 @@
         <v>88</v>
       </c>
       <c r="AU45" t="s" s="2">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="AV45" t="s" s="2">
         <v>88</v>
       </c>
       <c r="AW45" t="s" s="2">
-        <v>397</v>
+        <v>398</v>
       </c>
     </row>
     <row r="46" hidden="true">
       <c r="A46" t="s" s="2">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="E46" s="2"/>
       <c r="F46" t="s" s="2">
@@ -8638,16 +8639,16 @@
         <v>97</v>
       </c>
       <c r="K46" t="s" s="2">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="L46" t="s" s="2">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="M46" t="s" s="2">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="N46" t="s" s="2">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="O46" s="2"/>
       <c r="P46" t="s" s="2">
@@ -8697,7 +8698,7 @@
         <v>88</v>
       </c>
       <c r="AF46" t="s" s="2">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="AG46" t="s" s="2">
         <v>86</v>
@@ -8709,10 +8710,10 @@
         <v>88</v>
       </c>
       <c r="AJ46" t="s" s="2">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="AK46" t="s" s="2">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="AL46" t="s" s="2">
         <v>88</v>
@@ -8724,7 +8725,7 @@
         <v>88</v>
       </c>
       <c r="AO46" t="s" s="2">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="AP46" t="s" s="2">
         <v>88</v>
@@ -8733,7 +8734,7 @@
         <v>88</v>
       </c>
       <c r="AR46" t="s" s="2">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="AS46" t="s" s="2">
         <v>88</v>
@@ -8742,7 +8743,7 @@
         <v>88</v>
       </c>
       <c r="AU46" t="s" s="2">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="AV46" t="s" s="2">
         <v>88</v>
@@ -8753,10 +8754,10 @@
     </row>
     <row r="47" hidden="true">
       <c r="A47" t="s" s="2">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" t="s" s="2">
@@ -8892,10 +8893,10 @@
     </row>
     <row r="48" hidden="true">
       <c r="A48" t="s" s="2">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" t="s" s="2">
@@ -9033,14 +9034,14 @@
     </row>
     <row r="49" hidden="true">
       <c r="A49" t="s" s="2">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B49" t="s" s="2">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" t="s" s="2">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="E49" s="2"/>
       <c r="F49" t="s" s="2">
@@ -9065,7 +9066,7 @@
         <v>189</v>
       </c>
       <c r="M49" t="s" s="2">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="N49" t="s" s="2">
         <v>167</v>
@@ -9118,7 +9119,7 @@
         <v>88</v>
       </c>
       <c r="AF49" t="s" s="2">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="AG49" t="s" s="2">
         <v>86</v>
@@ -9174,10 +9175,10 @@
     </row>
     <row r="50" hidden="true">
       <c r="A50" t="s" s="2">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="B50" t="s" s="2">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="C50" s="2"/>
       <c r="D50" t="s" s="2">
@@ -9203,10 +9204,10 @@
         <v>181</v>
       </c>
       <c r="L50" t="s" s="2">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="M50" t="s" s="2">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="N50" s="2"/>
       <c r="O50" s="2"/>
@@ -9236,10 +9237,10 @@
         <v>245</v>
       </c>
       <c r="Y50" t="s" s="2">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="Z50" t="s" s="2">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="AA50" t="s" s="2">
         <v>88</v>
@@ -9257,7 +9258,7 @@
         <v>88</v>
       </c>
       <c r="AF50" t="s" s="2">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="AG50" t="s" s="2">
         <v>86</v>
@@ -9302,21 +9303,21 @@
         <v>88</v>
       </c>
       <c r="AU50" t="s" s="2">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="AV50" t="s" s="2">
         <v>88</v>
       </c>
       <c r="AW50" t="s" s="2">
-        <v>419</v>
+        <v>420</v>
       </c>
     </row>
     <row r="51" hidden="true">
       <c r="A51" t="s" s="2">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B51" t="s" s="2">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="C51" s="2"/>
       <c r="D51" t="s" s="2">
@@ -9452,10 +9453,10 @@
     </row>
     <row r="52" hidden="true">
       <c r="A52" t="s" s="2">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="B52" t="s" s="2">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="C52" s="2"/>
       <c r="D52" t="s" s="2">
@@ -9593,10 +9594,10 @@
     </row>
     <row r="53" hidden="true">
       <c r="A53" t="s" s="2">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="B53" t="s" s="2">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" t="s" s="2">
@@ -9668,7 +9669,7 @@
         <v>88</v>
       </c>
       <c r="AB53" t="s" s="2">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="AC53" s="2"/>
       <c r="AD53" t="s" s="2">
@@ -9678,7 +9679,7 @@
         <v>145</v>
       </c>
       <c r="AF53" t="s" s="2">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="AG53" t="s" s="2">
         <v>86</v>
@@ -9723,27 +9724,27 @@
         <v>88</v>
       </c>
       <c r="AU53" t="s" s="2">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="AV53" t="s" s="2">
         <v>88</v>
       </c>
       <c r="AW53" t="s" s="2">
-        <v>280</v>
+        <v>281</v>
       </c>
     </row>
     <row r="54" hidden="true">
       <c r="A54" t="s" s="2">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="B54" t="s" s="2">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="C54" t="s" s="2">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="D54" t="s" s="2">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="E54" s="2"/>
       <c r="F54" t="s" s="2">
@@ -9765,10 +9766,10 @@
         <v>272</v>
       </c>
       <c r="L54" t="s" s="2">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="M54" t="s" s="2">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="N54" t="s" s="2">
         <v>275</v>
@@ -9803,7 +9804,7 @@
       </c>
       <c r="Y54" s="2"/>
       <c r="Z54" t="s" s="2">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="AA54" t="s" s="2">
         <v>88</v>
@@ -9821,7 +9822,7 @@
         <v>88</v>
       </c>
       <c r="AF54" t="s" s="2">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="AG54" t="s" s="2">
         <v>86</v>
@@ -9842,7 +9843,7 @@
         <v>88</v>
       </c>
       <c r="AM54" t="s" s="2">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="AN54" t="s" s="2">
         <v>88</v>
@@ -9854,7 +9855,7 @@
         <v>88</v>
       </c>
       <c r="AQ54" t="s" s="2">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="AR54" t="s" s="2">
         <v>88</v>
@@ -9863,24 +9864,24 @@
         <v>88</v>
       </c>
       <c r="AT54" t="s" s="2">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="AU54" t="s" s="2">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="AV54" t="s" s="2">
         <v>88</v>
       </c>
       <c r="AW54" t="s" s="2">
-        <v>280</v>
+        <v>281</v>
       </c>
     </row>
     <row r="55" hidden="true">
       <c r="A55" t="s" s="2">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="B55" t="s" s="2">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="C55" s="2"/>
       <c r="D55" t="s" s="2">
@@ -9906,16 +9907,16 @@
         <v>157</v>
       </c>
       <c r="L55" t="s" s="2">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="M55" t="s" s="2">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="N55" t="s" s="2">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="O55" t="s" s="2">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="P55" t="s" s="2">
         <v>88</v>
@@ -9964,7 +9965,7 @@
         <v>88</v>
       </c>
       <c r="AF55" t="s" s="2">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="AG55" t="s" s="2">
         <v>86</v>
@@ -10009,21 +10010,21 @@
         <v>88</v>
       </c>
       <c r="AU55" t="s" s="2">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="AV55" t="s" s="2">
         <v>88</v>
       </c>
       <c r="AW55" t="s" s="2">
-        <v>341</v>
+        <v>342</v>
       </c>
     </row>
     <row r="56" hidden="true">
       <c r="A56" t="s" s="2">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="B56" t="s" s="2">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="C56" s="2"/>
       <c r="D56" t="s" s="2">
@@ -10046,17 +10047,17 @@
         <v>97</v>
       </c>
       <c r="K56" t="s" s="2">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="L56" t="s" s="2">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="M56" t="s" s="2">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="N56" s="2"/>
       <c r="O56" t="s" s="2">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="P56" t="s" s="2">
         <v>88</v>
@@ -10105,7 +10106,7 @@
         <v>88</v>
       </c>
       <c r="AF56" t="s" s="2">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="AG56" t="s" s="2">
         <v>96</v>
@@ -10150,21 +10151,21 @@
         <v>88</v>
       </c>
       <c r="AU56" t="s" s="2">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="AV56" t="s" s="2">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="AW56" t="s" s="2">
-        <v>439</v>
+        <v>440</v>
       </c>
     </row>
     <row r="57" hidden="true">
       <c r="A57" t="s" s="2">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="B57" t="s" s="2">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="C57" s="2"/>
       <c r="D57" t="s" s="2">
@@ -10300,10 +10301,10 @@
     </row>
     <row r="58" hidden="true">
       <c r="A58" t="s" s="2">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="B58" t="s" s="2">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="C58" s="2"/>
       <c r="D58" t="s" s="2">
@@ -10439,13 +10440,13 @@
     </row>
     <row r="59" hidden="true">
       <c r="A59" t="s" s="2">
+        <v>443</v>
+      </c>
+      <c r="B59" t="s" s="2">
         <v>442</v>
       </c>
-      <c r="B59" t="s" s="2">
-        <v>441</v>
-      </c>
       <c r="C59" t="s" s="2">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="D59" t="s" s="2">
         <v>88</v>
@@ -10467,13 +10468,13 @@
         <v>88</v>
       </c>
       <c r="K59" t="s" s="2">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="L59" t="s" s="2">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="M59" t="s" s="2">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="N59" s="2"/>
       <c r="O59" s="2"/>
@@ -10580,10 +10581,10 @@
     </row>
     <row r="60" hidden="true">
       <c r="A60" t="s" s="2">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="B60" t="s" s="2">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="C60" s="2"/>
       <c r="D60" t="s" s="2">
@@ -10609,13 +10610,13 @@
         <v>157</v>
       </c>
       <c r="L60" t="s" s="2">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="M60" t="s" s="2">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="N60" t="s" s="2">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="O60" s="2"/>
       <c r="P60" t="s" s="2">
@@ -10665,7 +10666,7 @@
         <v>88</v>
       </c>
       <c r="AF60" t="s" s="2">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="AG60" t="s" s="2">
         <v>86</v>
@@ -10674,7 +10675,7 @@
         <v>96</v>
       </c>
       <c r="AI60" t="s" s="2">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="AJ60" t="s" s="2">
         <v>88</v>
@@ -10721,10 +10722,10 @@
     </row>
     <row r="61" hidden="true">
       <c r="A61" t="s" s="2">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="B61" t="s" s="2">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="C61" s="2"/>
       <c r="D61" t="s" s="2">
@@ -10750,13 +10751,13 @@
         <v>193</v>
       </c>
       <c r="L61" t="s" s="2">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="M61" t="s" s="2">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="N61" t="s" s="2">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="O61" s="2"/>
       <c r="P61" t="s" s="2">
@@ -10806,7 +10807,7 @@
         <v>88</v>
       </c>
       <c r="AF61" t="s" s="2">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="AG61" t="s" s="2">
         <v>86</v>
@@ -10851,7 +10852,7 @@
         <v>88</v>
       </c>
       <c r="AU61" t="s" s="2">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="AV61" t="s" s="2">
         <v>88</v>
@@ -10862,10 +10863,10 @@
     </row>
     <row r="62" hidden="true">
       <c r="A62" t="s" s="2">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="B62" t="s" s="2">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="C62" s="2"/>
       <c r="D62" t="s" s="2">
@@ -10891,13 +10892,13 @@
         <v>157</v>
       </c>
       <c r="L62" t="s" s="2">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="M62" t="s" s="2">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="N62" t="s" s="2">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="O62" s="2"/>
       <c r="P62" t="s" s="2">
@@ -10947,7 +10948,7 @@
         <v>88</v>
       </c>
       <c r="AF62" t="s" s="2">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="AG62" t="s" s="2">
         <v>86</v>
@@ -11003,10 +11004,10 @@
     </row>
     <row r="63" hidden="true">
       <c r="A63" t="s" s="2">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="B63" t="s" s="2">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="C63" s="2"/>
       <c r="D63" t="s" s="2">
@@ -11029,17 +11030,17 @@
         <v>88</v>
       </c>
       <c r="K63" t="s" s="2">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="L63" t="s" s="2">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="M63" t="s" s="2">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="N63" s="2"/>
       <c r="O63" t="s" s="2">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="P63" t="s" s="2">
         <v>88</v>
@@ -11088,7 +11089,7 @@
         <v>88</v>
       </c>
       <c r="AF63" t="s" s="2">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="AG63" t="s" s="2">
         <v>86</v>
@@ -11133,7 +11134,7 @@
         <v>88</v>
       </c>
       <c r="AU63" t="s" s="2">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="AV63" t="s" s="2">
         <v>88</v>
@@ -11144,10 +11145,10 @@
     </row>
     <row r="64" hidden="true">
       <c r="A64" t="s" s="2">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="B64" t="s" s="2">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="C64" s="2"/>
       <c r="D64" t="s" s="2">
@@ -11170,17 +11171,17 @@
         <v>97</v>
       </c>
       <c r="K64" t="s" s="2">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="L64" t="s" s="2">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="M64" t="s" s="2">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="N64" s="2"/>
       <c r="O64" t="s" s="2">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="P64" t="s" s="2">
         <v>88</v>
@@ -11229,7 +11230,7 @@
         <v>88</v>
       </c>
       <c r="AF64" t="s" s="2">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="AG64" t="s" s="2">
         <v>86</v>
@@ -11274,10 +11275,10 @@
         <v>88</v>
       </c>
       <c r="AU64" t="s" s="2">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="AV64" t="s" s="2">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="AW64" t="s" s="2">
         <v>88</v>
@@ -11285,10 +11286,10 @@
     </row>
     <row r="65" hidden="true">
       <c r="A65" t="s" s="2">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="B65" t="s" s="2">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="C65" s="2"/>
       <c r="D65" t="s" s="2">
@@ -11424,10 +11425,10 @@
     </row>
     <row r="66" hidden="true">
       <c r="A66" t="s" s="2">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="B66" t="s" s="2">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="C66" s="2"/>
       <c r="D66" t="s" s="2">
@@ -11565,10 +11566,10 @@
     </row>
     <row r="67" hidden="true">
       <c r="A67" t="s" s="2">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="B67" t="s" s="2">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="C67" s="2"/>
       <c r="D67" t="s" s="2">
@@ -11594,13 +11595,13 @@
         <v>157</v>
       </c>
       <c r="L67" t="s" s="2">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="M67" t="s" s="2">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="N67" t="s" s="2">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="O67" s="2"/>
       <c r="P67" t="s" s="2">
@@ -11650,7 +11651,7 @@
         <v>88</v>
       </c>
       <c r="AF67" t="s" s="2">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="AG67" t="s" s="2">
         <v>86</v>
@@ -11659,7 +11660,7 @@
         <v>96</v>
       </c>
       <c r="AI67" t="s" s="2">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="AJ67" t="s" s="2">
         <v>88</v>
@@ -11706,10 +11707,10 @@
     </row>
     <row r="68" hidden="true">
       <c r="A68" t="s" s="2">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="B68" t="s" s="2">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="C68" s="2"/>
       <c r="D68" t="s" s="2">
@@ -11735,13 +11736,13 @@
         <v>193</v>
       </c>
       <c r="L68" t="s" s="2">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="M68" t="s" s="2">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="N68" t="s" s="2">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="O68" s="2"/>
       <c r="P68" t="s" s="2">
@@ -11791,7 +11792,7 @@
         <v>88</v>
       </c>
       <c r="AF68" t="s" s="2">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="AG68" t="s" s="2">
         <v>86</v>
@@ -11836,7 +11837,7 @@
         <v>88</v>
       </c>
       <c r="AU68" t="s" s="2">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="AV68" t="s" s="2">
         <v>88</v>
@@ -11847,10 +11848,10 @@
     </row>
     <row r="69" hidden="true">
       <c r="A69" t="s" s="2">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="B69" t="s" s="2">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="C69" s="2"/>
       <c r="D69" t="s" s="2">
@@ -11876,13 +11877,13 @@
         <v>157</v>
       </c>
       <c r="L69" t="s" s="2">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="M69" t="s" s="2">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="N69" t="s" s="2">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="O69" s="2"/>
       <c r="P69" t="s" s="2">
@@ -11932,7 +11933,7 @@
         <v>88</v>
       </c>
       <c r="AF69" t="s" s="2">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="AG69" t="s" s="2">
         <v>86</v>
@@ -11988,10 +11989,10 @@
     </row>
     <row r="70" hidden="true">
       <c r="A70" t="s" s="2">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="B70" t="s" s="2">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="C70" s="2"/>
       <c r="D70" t="s" s="2">
@@ -12017,10 +12018,10 @@
         <v>181</v>
       </c>
       <c r="L70" t="s" s="2">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="M70" t="s" s="2">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="N70" s="2"/>
       <c r="O70" s="2"/>
@@ -12050,10 +12051,10 @@
         <v>245</v>
       </c>
       <c r="Y70" t="s" s="2">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="Z70" t="s" s="2">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="AA70" t="s" s="2">
         <v>88</v>
@@ -12071,7 +12072,7 @@
         <v>88</v>
       </c>
       <c r="AF70" t="s" s="2">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="AG70" t="s" s="2">
         <v>86</v>
@@ -12116,10 +12117,10 @@
         <v>88</v>
       </c>
       <c r="AU70" t="s" s="2">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="AV70" t="s" s="2">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="AW70" t="s" s="2">
         <v>88</v>
@@ -12127,14 +12128,14 @@
     </row>
     <row r="71" hidden="true">
       <c r="A71" t="s" s="2">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="B71" t="s" s="2">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="C71" s="2"/>
       <c r="D71" t="s" s="2">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="E71" s="2"/>
       <c r="F71" t="s" s="2">
@@ -12153,16 +12154,16 @@
         <v>97</v>
       </c>
       <c r="K71" t="s" s="2">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="L71" t="s" s="2">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="M71" t="s" s="2">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="N71" t="s" s="2">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="O71" s="2"/>
       <c r="P71" t="s" s="2">
@@ -12212,7 +12213,7 @@
         <v>88</v>
       </c>
       <c r="AF71" t="s" s="2">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="AG71" t="s" s="2">
         <v>86</v>
@@ -12227,7 +12228,7 @@
         <v>88</v>
       </c>
       <c r="AK71" t="s" s="2">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="AL71" t="s" s="2">
         <v>88</v>
@@ -12239,7 +12240,7 @@
         <v>88</v>
       </c>
       <c r="AO71" t="s" s="2">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="AP71" t="s" s="2">
         <v>88</v>
@@ -12248,7 +12249,7 @@
         <v>88</v>
       </c>
       <c r="AR71" t="s" s="2">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="AS71" t="s" s="2">
         <v>88</v>
@@ -12257,10 +12258,10 @@
         <v>88</v>
       </c>
       <c r="AU71" t="s" s="2">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="AV71" t="s" s="2">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="AW71" t="s" s="2">
         <v>88</v>
@@ -12268,14 +12269,14 @@
     </row>
     <row r="72" hidden="true">
       <c r="A72" t="s" s="2">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="B72" t="s" s="2">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="C72" s="2"/>
       <c r="D72" t="s" s="2">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="E72" s="2"/>
       <c r="F72" t="s" s="2">
@@ -12297,10 +12298,10 @@
         <v>181</v>
       </c>
       <c r="L72" t="s" s="2">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="M72" t="s" s="2">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="N72" s="2"/>
       <c r="O72" s="2"/>
@@ -12330,10 +12331,10 @@
         <v>119</v>
       </c>
       <c r="Y72" t="s" s="2">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="Z72" t="s" s="2">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="AA72" t="s" s="2">
         <v>88</v>
@@ -12351,7 +12352,7 @@
         <v>88</v>
       </c>
       <c r="AF72" t="s" s="2">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="AG72" t="s" s="2">
         <v>86</v>
@@ -12366,7 +12367,7 @@
         <v>88</v>
       </c>
       <c r="AK72" t="s" s="2">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="AL72" t="s" s="2">
         <v>88</v>
@@ -12378,7 +12379,7 @@
         <v>88</v>
       </c>
       <c r="AO72" t="s" s="2">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="AP72" t="s" s="2">
         <v>88</v>
@@ -12387,7 +12388,7 @@
         <v>88</v>
       </c>
       <c r="AR72" t="s" s="2">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="AS72" t="s" s="2">
         <v>88</v>
@@ -12396,21 +12397,21 @@
         <v>88</v>
       </c>
       <c r="AU72" t="s" s="2">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="AV72" t="s" s="2">
         <v>88</v>
       </c>
       <c r="AW72" t="s" s="2">
-        <v>503</v>
+        <v>504</v>
       </c>
     </row>
     <row r="73" hidden="true">
       <c r="A73" t="s" s="2">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="B73" t="s" s="2">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="C73" s="2"/>
       <c r="D73" t="s" s="2">
@@ -12546,10 +12547,10 @@
     </row>
     <row r="74" hidden="true">
       <c r="A74" t="s" s="2">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="B74" t="s" s="2">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="C74" s="2"/>
       <c r="D74" t="s" s="2">
@@ -12685,13 +12686,13 @@
     </row>
     <row r="75" hidden="true">
       <c r="A75" t="s" s="2">
+        <v>507</v>
+      </c>
+      <c r="B75" t="s" s="2">
         <v>506</v>
       </c>
-      <c r="B75" t="s" s="2">
-        <v>505</v>
-      </c>
       <c r="C75" t="s" s="2">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="D75" t="s" s="2">
         <v>88</v>
@@ -12713,13 +12714,13 @@
         <v>88</v>
       </c>
       <c r="K75" t="s" s="2">
+        <v>509</v>
+      </c>
+      <c r="L75" t="s" s="2">
         <v>508</v>
       </c>
-      <c r="L75" t="s" s="2">
-        <v>507</v>
-      </c>
       <c r="M75" t="s" s="2">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="N75" s="2"/>
       <c r="O75" s="2"/>
@@ -12826,10 +12827,10 @@
     </row>
     <row r="76" hidden="true">
       <c r="A76" t="s" s="2">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="B76" t="s" s="2">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="C76" s="2"/>
       <c r="D76" t="s" s="2">
@@ -12965,10 +12966,10 @@
     </row>
     <row r="77" hidden="true">
       <c r="A77" t="s" s="2">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="B77" t="s" s="2">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="C77" s="2"/>
       <c r="D77" t="s" s="2">
@@ -13106,10 +13107,10 @@
     </row>
     <row r="78" hidden="true">
       <c r="A78" t="s" s="2">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="B78" t="s" s="2">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="C78" s="2"/>
       <c r="D78" t="s" s="2">
@@ -13149,7 +13150,7 @@
       </c>
       <c r="Q78" s="2"/>
       <c r="R78" t="s" s="2">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="S78" t="s" s="2">
         <v>88</v>
@@ -13247,10 +13248,10 @@
     </row>
     <row r="79" hidden="true">
       <c r="A79" t="s" s="2">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="B79" t="s" s="2">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="C79" s="2"/>
       <c r="D79" t="s" s="2">
@@ -13276,10 +13277,10 @@
         <v>181</v>
       </c>
       <c r="L79" t="s" s="2">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="M79" t="s" s="2">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="N79" s="2"/>
       <c r="O79" s="2"/>
@@ -13318,14 +13319,14 @@
         <v>88</v>
       </c>
       <c r="AB79" t="s" s="2">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="AC79" s="2"/>
       <c r="AD79" t="s" s="2">
         <v>88</v>
       </c>
       <c r="AE79" t="s" s="2">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="AF79" t="s" s="2">
         <v>186</v>
@@ -13384,10 +13385,10 @@
     </row>
     <row r="80" hidden="true">
       <c r="A80" t="s" s="2">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="B80" t="s" s="2">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="C80" t="s" s="2">
         <v>179</v>
@@ -13415,10 +13416,10 @@
         <v>181</v>
       </c>
       <c r="L80" t="s" s="2">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="M80" t="s" s="2">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="N80" s="2"/>
       <c r="O80" s="2"/>
@@ -13448,10 +13449,10 @@
         <v>119</v>
       </c>
       <c r="Y80" t="s" s="2">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="Z80" t="s" s="2">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="AA80" t="s" s="2">
         <v>88</v>
@@ -13484,7 +13485,7 @@
         <v>88</v>
       </c>
       <c r="AK80" t="s" s="2">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="AL80" t="s" s="2">
         <v>88</v>
@@ -13525,10 +13526,10 @@
     </row>
     <row r="81" hidden="true">
       <c r="A81" t="s" s="2">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="B81" t="s" s="2">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="C81" s="2"/>
       <c r="D81" t="s" s="2">
@@ -13612,7 +13613,7 @@
         <v>88</v>
       </c>
       <c r="AF81" t="s" s="2">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="AG81" t="s" s="2">
         <v>86</v>
@@ -13657,21 +13658,21 @@
         <v>88</v>
       </c>
       <c r="AU81" t="s" s="2">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="AV81" t="s" s="2">
         <v>88</v>
       </c>
       <c r="AW81" t="s" s="2">
-        <v>280</v>
+        <v>281</v>
       </c>
     </row>
     <row r="82" hidden="true">
       <c r="A82" t="s" s="2">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="B82" t="s" s="2">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="C82" s="2"/>
       <c r="D82" t="s" s="2">
@@ -13697,16 +13698,16 @@
         <v>157</v>
       </c>
       <c r="L82" t="s" s="2">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="M82" t="s" s="2">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="N82" t="s" s="2">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="O82" t="s" s="2">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="P82" t="s" s="2">
         <v>88</v>
@@ -13755,7 +13756,7 @@
         <v>88</v>
       </c>
       <c r="AF82" t="s" s="2">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="AG82" t="s" s="2">
         <v>86</v>
@@ -13800,21 +13801,21 @@
         <v>88</v>
       </c>
       <c r="AU82" t="s" s="2">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="AV82" t="s" s="2">
         <v>88</v>
       </c>
       <c r="AW82" t="s" s="2">
-        <v>341</v>
+        <v>342</v>
       </c>
     </row>
     <row r="83" hidden="true">
       <c r="A83" t="s" s="2">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="B83" t="s" s="2">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="C83" s="2"/>
       <c r="D83" t="s" s="2">
@@ -13840,13 +13841,13 @@
         <v>181</v>
       </c>
       <c r="L83" t="s" s="2">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="M83" t="s" s="2">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="N83" t="s" s="2">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="O83" s="2"/>
       <c r="P83" t="s" s="2">
@@ -13875,10 +13876,10 @@
         <v>245</v>
       </c>
       <c r="Y83" t="s" s="2">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="Z83" t="s" s="2">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="AA83" t="s" s="2">
         <v>88</v>
@@ -13896,7 +13897,7 @@
         <v>88</v>
       </c>
       <c r="AF83" t="s" s="2">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="AG83" t="s" s="2">
         <v>86</v>
@@ -13941,7 +13942,7 @@
         <v>88</v>
       </c>
       <c r="AU83" t="s" s="2">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="AV83" t="s" s="2">
         <v>88</v>
@@ -13952,10 +13953,10 @@
     </row>
     <row r="84" hidden="true">
       <c r="A84" t="s" s="2">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="B84" t="s" s="2">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="C84" s="2"/>
       <c r="D84" t="s" s="2">
@@ -13978,16 +13979,16 @@
         <v>88</v>
       </c>
       <c r="K84" t="s" s="2">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="L84" t="s" s="2">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="M84" t="s" s="2">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="N84" t="s" s="2">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="O84" s="2"/>
       <c r="P84" t="s" s="2">
@@ -14037,7 +14038,7 @@
         <v>88</v>
       </c>
       <c r="AF84" t="s" s="2">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="AG84" t="s" s="2">
         <v>86</v>
@@ -14055,7 +14056,7 @@
         <v>88</v>
       </c>
       <c r="AL84" t="s" s="2">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="AM84" t="s" s="2">
         <v>88</v>
@@ -14067,7 +14068,7 @@
         <v>88</v>
       </c>
       <c r="AP84" t="s" s="2">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="AQ84" t="s" s="2">
         <v>88</v>
@@ -14076,13 +14077,13 @@
         <v>88</v>
       </c>
       <c r="AS84" t="s" s="2">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="AT84" t="s" s="2">
         <v>88</v>
       </c>
       <c r="AU84" t="s" s="2">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="AV84" t="s" s="2">
         <v>88</v>
@@ -14093,10 +14094,10 @@
     </row>
     <row r="85" hidden="true">
       <c r="A85" t="s" s="2">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="B85" t="s" s="2">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="C85" s="2"/>
       <c r="D85" t="s" s="2">
@@ -14122,13 +14123,13 @@
         <v>181</v>
       </c>
       <c r="L85" t="s" s="2">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="M85" t="s" s="2">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="N85" t="s" s="2">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="O85" s="2"/>
       <c r="P85" t="s" s="2">
@@ -14157,10 +14158,10 @@
         <v>245</v>
       </c>
       <c r="Y85" t="s" s="2">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="Z85" t="s" s="2">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="AA85" t="s" s="2">
         <v>88</v>
@@ -14178,7 +14179,7 @@
         <v>88</v>
       </c>
       <c r="AF85" t="s" s="2">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="AG85" t="s" s="2">
         <v>86</v>
@@ -14223,7 +14224,7 @@
         <v>88</v>
       </c>
       <c r="AU85" t="s" s="2">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="AV85" t="s" s="2">
         <v>88</v>
@@ -14234,10 +14235,10 @@
     </row>
     <row r="86" hidden="true">
       <c r="A86" t="s" s="2">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="B86" t="s" s="2">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="C86" s="2"/>
       <c r="D86" t="s" s="2">
@@ -14260,17 +14261,17 @@
         <v>88</v>
       </c>
       <c r="K86" t="s" s="2">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="L86" t="s" s="2">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="M86" t="s" s="2">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="N86" s="2"/>
       <c r="O86" t="s" s="2">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="P86" t="s" s="2">
         <v>88</v>
@@ -14319,7 +14320,7 @@
         <v>88</v>
       </c>
       <c r="AF86" t="s" s="2">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="AG86" t="s" s="2">
         <v>86</v>
@@ -14364,7 +14365,7 @@
         <v>88</v>
       </c>
       <c r="AU86" t="s" s="2">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="AV86" t="s" s="2">
         <v>88</v>
@@ -14375,10 +14376,10 @@
     </row>
     <row r="87" hidden="true">
       <c r="A87" t="s" s="2">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="B87" t="s" s="2">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="C87" s="2"/>
       <c r="D87" t="s" s="2">
@@ -14404,10 +14405,10 @@
         <v>181</v>
       </c>
       <c r="L87" t="s" s="2">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="M87" t="s" s="2">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="N87" s="2"/>
       <c r="O87" s="2"/>
@@ -14437,10 +14438,10 @@
         <v>245</v>
       </c>
       <c r="Y87" t="s" s="2">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="Z87" t="s" s="2">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="AA87" t="s" s="2">
         <v>88</v>
@@ -14458,7 +14459,7 @@
         <v>88</v>
       </c>
       <c r="AF87" t="s" s="2">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="AG87" t="s" s="2">
         <v>86</v>
@@ -14503,7 +14504,7 @@
         <v>88</v>
       </c>
       <c r="AU87" t="s" s="2">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="AV87" t="s" s="2">
         <v>88</v>
@@ -14514,10 +14515,10 @@
     </row>
     <row r="88" hidden="true">
       <c r="A88" t="s" s="2">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="B88" t="s" s="2">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="C88" s="2"/>
       <c r="D88" t="s" s="2">
@@ -14540,13 +14541,13 @@
         <v>88</v>
       </c>
       <c r="K88" t="s" s="2">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="L88" t="s" s="2">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="M88" t="s" s="2">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="N88" s="2"/>
       <c r="O88" s="2"/>
@@ -14597,7 +14598,7 @@
         <v>88</v>
       </c>
       <c r="AF88" t="s" s="2">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="AG88" t="s" s="2">
         <v>86</v>
@@ -14642,21 +14643,21 @@
         <v>88</v>
       </c>
       <c r="AU88" t="s" s="2">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="AV88" t="s" s="2">
         <v>88</v>
       </c>
       <c r="AW88" t="s" s="2">
-        <v>566</v>
+        <v>567</v>
       </c>
     </row>
     <row r="89" hidden="true">
       <c r="A89" t="s" s="2">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="B89" t="s" s="2">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="C89" s="2"/>
       <c r="D89" t="s" s="2">
@@ -14679,13 +14680,13 @@
         <v>88</v>
       </c>
       <c r="K89" t="s" s="2">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="L89" t="s" s="2">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="M89" t="s" s="2">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="N89" s="2"/>
       <c r="O89" s="2"/>
@@ -14736,7 +14737,7 @@
         <v>88</v>
       </c>
       <c r="AF89" t="s" s="2">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="AG89" t="s" s="2">
         <v>86</v>
@@ -14748,7 +14749,7 @@
         <v>88</v>
       </c>
       <c r="AJ89" t="s" s="2">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="AK89" t="s" s="2">
         <v>88</v>
@@ -14781,7 +14782,7 @@
         <v>88</v>
       </c>
       <c r="AU89" t="s" s="2">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="AV89" t="s" s="2">
         <v>88</v>
@@ -14792,10 +14793,10 @@
     </row>
     <row r="90" hidden="true">
       <c r="A90" t="s" s="2">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="B90" t="s" s="2">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="C90" s="2"/>
       <c r="D90" t="s" s="2">
@@ -14931,10 +14932,10 @@
     </row>
     <row r="91" hidden="true">
       <c r="A91" t="s" s="2">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="B91" t="s" s="2">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="C91" s="2"/>
       <c r="D91" t="s" s="2">
@@ -15072,14 +15073,14 @@
     </row>
     <row r="92" hidden="true">
       <c r="A92" t="s" s="2">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="B92" t="s" s="2">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="C92" s="2"/>
       <c r="D92" t="s" s="2">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="E92" s="2"/>
       <c r="F92" t="s" s="2">
@@ -15104,7 +15105,7 @@
         <v>189</v>
       </c>
       <c r="M92" t="s" s="2">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="N92" t="s" s="2">
         <v>167</v>
@@ -15157,7 +15158,7 @@
         <v>88</v>
       </c>
       <c r="AF92" t="s" s="2">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="AG92" t="s" s="2">
         <v>86</v>
@@ -15213,10 +15214,10 @@
     </row>
     <row r="93" hidden="true">
       <c r="A93" t="s" s="2">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="B93" t="s" s="2">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="C93" s="2"/>
       <c r="D93" t="s" s="2">
@@ -15242,10 +15243,10 @@
         <v>181</v>
       </c>
       <c r="L93" t="s" s="2">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="M93" t="s" s="2">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="N93" s="2"/>
       <c r="O93" s="2"/>
@@ -15272,13 +15273,13 @@
         <v>88</v>
       </c>
       <c r="X93" t="s" s="2">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="Y93" t="s" s="2">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="Z93" t="s" s="2">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="AA93" t="s" s="2">
         <v>88</v>
@@ -15296,7 +15297,7 @@
         <v>88</v>
       </c>
       <c r="AF93" t="s" s="2">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="AG93" t="s" s="2">
         <v>86</v>
@@ -15341,7 +15342,7 @@
         <v>88</v>
       </c>
       <c r="AU93" t="s" s="2">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="AV93" t="s" s="2">
         <v>88</v>
@@ -15352,14 +15353,14 @@
     </row>
     <row r="94" hidden="true">
       <c r="A94" t="s" s="2">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="B94" t="s" s="2">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="C94" s="2"/>
       <c r="D94" t="s" s="2">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E94" s="2"/>
       <c r="F94" t="s" s="2">
@@ -15378,13 +15379,13 @@
         <v>88</v>
       </c>
       <c r="K94" t="s" s="2">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="L94" t="s" s="2">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="M94" t="s" s="2">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="N94" s="2"/>
       <c r="O94" s="2"/>
@@ -15435,7 +15436,7 @@
         <v>88</v>
       </c>
       <c r="AF94" t="s" s="2">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="AG94" t="s" s="2">
         <v>96</v>
@@ -15450,7 +15451,7 @@
         <v>88</v>
       </c>
       <c r="AK94" t="s" s="2">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="AL94" t="s" s="2">
         <v>88</v>
@@ -15462,7 +15463,7 @@
         <v>88</v>
       </c>
       <c r="AO94" t="s" s="2">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="AP94" t="s" s="2">
         <v>88</v>
@@ -15471,7 +15472,7 @@
         <v>88</v>
       </c>
       <c r="AR94" t="s" s="2">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="AS94" t="s" s="2">
         <v>88</v>
@@ -15480,7 +15481,7 @@
         <v>88</v>
       </c>
       <c r="AU94" t="s" s="2">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="AV94" t="s" s="2">
         <v>88</v>
@@ -15491,10 +15492,10 @@
     </row>
     <row r="95" hidden="true">
       <c r="A95" t="s" s="2">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="B95" t="s" s="2">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="C95" s="2"/>
       <c r="D95" t="s" s="2">
@@ -15517,19 +15518,19 @@
         <v>88</v>
       </c>
       <c r="K95" t="s" s="2">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="L95" t="s" s="2">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="M95" t="s" s="2">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="N95" t="s" s="2">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="O95" t="s" s="2">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="P95" t="s" s="2">
         <v>88</v>
@@ -15578,7 +15579,7 @@
         <v>88</v>
       </c>
       <c r="AF95" t="s" s="2">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="AG95" t="s" s="2">
         <v>86</v>
@@ -15623,7 +15624,7 @@
         <v>88</v>
       </c>
       <c r="AU95" t="s" s="2">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="AV95" t="s" s="2">
         <v>88</v>
@@ -15634,10 +15635,10 @@
     </row>
     <row r="96" hidden="true">
       <c r="A96" t="s" s="2">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="B96" t="s" s="2">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="C96" s="2"/>
       <c r="D96" t="s" s="2">
@@ -15663,13 +15664,13 @@
         <v>181</v>
       </c>
       <c r="L96" t="s" s="2">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="M96" t="s" s="2">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="N96" t="s" s="2">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="O96" s="2"/>
       <c r="P96" t="s" s="2">
@@ -15698,10 +15699,10 @@
         <v>245</v>
       </c>
       <c r="Y96" t="s" s="2">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="Z96" t="s" s="2">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="AA96" t="s" s="2">
         <v>88</v>
@@ -15719,7 +15720,7 @@
         <v>88</v>
       </c>
       <c r="AF96" t="s" s="2">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="AG96" t="s" s="2">
         <v>86</v>
@@ -15764,7 +15765,7 @@
         <v>88</v>
       </c>
       <c r="AU96" t="s" s="2">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="AV96" t="s" s="2">
         <v>88</v>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@0f59f6a13c621beb4fe972ff593b4605a78dcdbd 🚀
</commit_message>
<xml_diff>
--- a/StructureDefinition-Procedure.xlsx
+++ b/StructureDefinition-Procedure.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4339" uniqueCount="602">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4341" uniqueCount="603">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-03-24T11:37:37+00:00</t>
+    <t>2025-04-01T10:33:26+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -590,6 +590,10 @@
   </si>
   <si>
     <t>The method or technique that was used to perform the procedure, e.g. approach, lavage, pressuring, ets.</t>
+  </si>
+  <si>
+    <t>HCIM Procedure allows for the possiblity to define multiple procedure methods, but this core extension restricts this to just a single method, resulting in a cardinality mismatch with the zib. It is advised to use the most important procedure method in this extension.
+This issue will be fixed in the next version of this profile.</t>
   </si>
   <si>
     <t>VerrichtingMethodeCodelijst</t>
@@ -4149,7 +4153,9 @@
       <c r="M14" t="s" s="2">
         <v>183</v>
       </c>
-      <c r="N14" s="2"/>
+      <c r="N14" t="s" s="2">
+        <v>184</v>
+      </c>
       <c r="O14" s="2"/>
       <c r="P14" t="s" s="2">
         <v>88</v>
@@ -4177,10 +4183,10 @@
         <v>119</v>
       </c>
       <c r="Y14" t="s" s="2">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="Z14" t="s" s="2">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="AA14" t="s" s="2">
         <v>88</v>
@@ -4198,7 +4204,7 @@
         <v>88</v>
       </c>
       <c r="AF14" t="s" s="2">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="AG14" t="s" s="2">
         <v>86</v>
@@ -4213,7 +4219,7 @@
         <v>88</v>
       </c>
       <c r="AK14" t="s" s="2">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="AL14" t="s" s="2">
         <v>88</v>
@@ -4254,10 +4260,10 @@
     </row>
     <row r="15" hidden="true">
       <c r="A15" t="s" s="2">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B15" t="s" s="2">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" t="s" s="2">
@@ -4283,10 +4289,10 @@
         <v>141</v>
       </c>
       <c r="L15" t="s" s="2">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="M15" t="s" s="2">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="N15" t="s" s="2">
         <v>167</v>
@@ -4339,7 +4345,7 @@
         <v>88</v>
       </c>
       <c r="AF15" t="s" s="2">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="AG15" t="s" s="2">
         <v>86</v>
@@ -4395,10 +4401,10 @@
     </row>
     <row r="16" hidden="true">
       <c r="A16" t="s" s="2">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" t="s" s="2">
@@ -4421,17 +4427,17 @@
         <v>97</v>
       </c>
       <c r="K16" t="s" s="2">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="L16" t="s" s="2">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="M16" t="s" s="2">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="N16" s="2"/>
       <c r="O16" t="s" s="2">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="P16" t="s" s="2">
         <v>88</v>
@@ -4480,7 +4486,7 @@
         <v>88</v>
       </c>
       <c r="AF16" t="s" s="2">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="AG16" t="s" s="2">
         <v>86</v>
@@ -4504,7 +4510,7 @@
         <v>88</v>
       </c>
       <c r="AN16" t="s" s="2">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="AO16" t="s" s="2">
         <v>88</v>
@@ -4525,21 +4531,21 @@
         <v>88</v>
       </c>
       <c r="AU16" t="s" s="2">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="AV16" t="s" s="2">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="AW16" t="s" s="2">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="17" hidden="true">
       <c r="A17" t="s" s="2">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" t="s" s="2">
@@ -4562,13 +4568,13 @@
         <v>97</v>
       </c>
       <c r="K17" t="s" s="2">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="L17" t="s" s="2">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="M17" t="s" s="2">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="N17" s="2"/>
       <c r="O17" s="2"/>
@@ -4619,7 +4625,7 @@
         <v>88</v>
       </c>
       <c r="AF17" t="s" s="2">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="AG17" t="s" s="2">
         <v>86</v>
@@ -4664,7 +4670,7 @@
         <v>88</v>
       </c>
       <c r="AU17" t="s" s="2">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AV17" t="s" s="2">
         <v>88</v>
@@ -4675,14 +4681,14 @@
     </row>
     <row r="18" hidden="true">
       <c r="A18" t="s" s="2">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B18" t="s" s="2">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" t="s" s="2">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="E18" s="2"/>
       <c r="F18" t="s" s="2">
@@ -4701,13 +4707,13 @@
         <v>97</v>
       </c>
       <c r="K18" t="s" s="2">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="L18" t="s" s="2">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="M18" t="s" s="2">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="N18" s="2"/>
       <c r="O18" s="2"/>
@@ -4746,7 +4752,7 @@
         <v>88</v>
       </c>
       <c r="AB18" t="s" s="2">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="AC18" s="2"/>
       <c r="AD18" t="s" s="2">
@@ -4756,7 +4762,7 @@
         <v>145</v>
       </c>
       <c r="AF18" t="s" s="2">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AG18" t="s" s="2">
         <v>86</v>
@@ -4801,7 +4807,7 @@
         <v>88</v>
       </c>
       <c r="AU18" t="s" s="2">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AV18" t="s" s="2">
         <v>88</v>
@@ -4812,16 +4818,16 @@
     </row>
     <row r="19" hidden="true">
       <c r="A19" t="s" s="2">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C19" t="s" s="2">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D19" t="s" s="2">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="E19" s="2"/>
       <c r="F19" t="s" s="2">
@@ -4840,16 +4846,16 @@
         <v>97</v>
       </c>
       <c r="K19" t="s" s="2">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="L19" t="s" s="2">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="M19" t="s" s="2">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="N19" t="s" s="2">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="O19" s="2"/>
       <c r="P19" t="s" s="2">
@@ -4899,7 +4905,7 @@
         <v>88</v>
       </c>
       <c r="AF19" t="s" s="2">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AG19" t="s" s="2">
         <v>86</v>
@@ -4914,7 +4920,7 @@
         <v>88</v>
       </c>
       <c r="AK19" t="s" s="2">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="AL19" t="s" s="2">
         <v>88</v>
@@ -4926,7 +4932,7 @@
         <v>88</v>
       </c>
       <c r="AO19" t="s" s="2">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="AP19" t="s" s="2">
         <v>88</v>
@@ -4935,7 +4941,7 @@
         <v>88</v>
       </c>
       <c r="AR19" t="s" s="2">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="AS19" t="s" s="2">
         <v>88</v>
@@ -4944,7 +4950,7 @@
         <v>88</v>
       </c>
       <c r="AU19" t="s" s="2">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AV19" t="s" s="2">
         <v>88</v>
@@ -4955,14 +4961,14 @@
     </row>
     <row r="20" hidden="true">
       <c r="A20" t="s" s="2">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" t="s" s="2">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E20" s="2"/>
       <c r="F20" t="s" s="2">
@@ -4981,16 +4987,16 @@
         <v>97</v>
       </c>
       <c r="K20" t="s" s="2">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="L20" t="s" s="2">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="M20" t="s" s="2">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="N20" t="s" s="2">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="O20" s="2"/>
       <c r="P20" t="s" s="2">
@@ -5040,7 +5046,7 @@
         <v>88</v>
       </c>
       <c r="AF20" t="s" s="2">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="AG20" t="s" s="2">
         <v>86</v>
@@ -5085,7 +5091,7 @@
         <v>88</v>
       </c>
       <c r="AU20" t="s" s="2">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="AV20" t="s" s="2">
         <v>88</v>
@@ -5096,10 +5102,10 @@
     </row>
     <row r="21" hidden="true">
       <c r="A21" t="s" s="2">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" t="s" s="2">
@@ -5125,13 +5131,13 @@
         <v>115</v>
       </c>
       <c r="L21" t="s" s="2">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="M21" t="s" s="2">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="N21" t="s" s="2">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="O21" s="2"/>
       <c r="P21" t="s" s="2">
@@ -5157,13 +5163,13 @@
         <v>88</v>
       </c>
       <c r="X21" t="s" s="2">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="Y21" t="s" s="2">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="Z21" t="s" s="2">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="AA21" t="s" s="2">
         <v>88</v>
@@ -5181,7 +5187,7 @@
         <v>88</v>
       </c>
       <c r="AF21" t="s" s="2">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="AG21" t="s" s="2">
         <v>96</v>
@@ -5226,10 +5232,10 @@
         <v>88</v>
       </c>
       <c r="AU21" t="s" s="2">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AV21" t="s" s="2">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="AW21" t="s" s="2">
         <v>88</v>
@@ -5237,10 +5243,10 @@
     </row>
     <row r="22" hidden="true">
       <c r="A22" t="s" s="2">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" t="s" s="2">
@@ -5263,16 +5269,16 @@
         <v>97</v>
       </c>
       <c r="K22" t="s" s="2">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="L22" t="s" s="2">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="M22" t="s" s="2">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="N22" t="s" s="2">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="O22" s="2"/>
       <c r="P22" t="s" s="2">
@@ -5322,7 +5328,7 @@
         <v>88</v>
       </c>
       <c r="AF22" t="s" s="2">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="AG22" t="s" s="2">
         <v>86</v>
@@ -5367,7 +5373,7 @@
         <v>88</v>
       </c>
       <c r="AU22" t="s" s="2">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="AV22" t="s" s="2">
         <v>88</v>
@@ -5378,10 +5384,10 @@
     </row>
     <row r="23" hidden="true">
       <c r="A23" t="s" s="2">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" t="s" s="2">
@@ -5407,10 +5413,10 @@
         <v>181</v>
       </c>
       <c r="L23" t="s" s="2">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="M23" t="s" s="2">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="N23" s="2"/>
       <c r="O23" s="2"/>
@@ -5437,13 +5443,13 @@
         <v>88</v>
       </c>
       <c r="X23" t="s" s="2">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="Y23" t="s" s="2">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="Z23" t="s" s="2">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="AA23" t="s" s="2">
         <v>88</v>
@@ -5461,7 +5467,7 @@
         <v>88</v>
       </c>
       <c r="AF23" t="s" s="2">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AG23" t="s" s="2">
         <v>86</v>
@@ -5470,7 +5476,7 @@
         <v>96</v>
       </c>
       <c r="AI23" t="s" s="2">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="AJ23" t="s" s="2">
         <v>88</v>
@@ -5506,7 +5512,7 @@
         <v>88</v>
       </c>
       <c r="AU23" t="s" s="2">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="AV23" t="s" s="2">
         <v>88</v>
@@ -5517,10 +5523,10 @@
     </row>
     <row r="24" hidden="true">
       <c r="A24" t="s" s="2">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
@@ -5546,10 +5552,10 @@
         <v>181</v>
       </c>
       <c r="L24" t="s" s="2">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="M24" t="s" s="2">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="N24" s="2"/>
       <c r="O24" s="2"/>
@@ -5564,7 +5570,7 @@
         <v>88</v>
       </c>
       <c r="T24" t="s" s="2">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="U24" t="s" s="2">
         <v>88</v>
@@ -5576,13 +5582,13 @@
         <v>88</v>
       </c>
       <c r="X24" t="s" s="2">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="Y24" t="s" s="2">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="Z24" t="s" s="2">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AA24" t="s" s="2">
         <v>88</v>
@@ -5600,7 +5606,7 @@
         <v>88</v>
       </c>
       <c r="AF24" t="s" s="2">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="AG24" t="s" s="2">
         <v>86</v>
@@ -5645,10 +5651,10 @@
         <v>88</v>
       </c>
       <c r="AU24" t="s" s="2">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="AV24" t="s" s="2">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="AW24" t="s" s="2">
         <v>88</v>
@@ -5656,14 +5662,14 @@
     </row>
     <row r="25" hidden="true">
       <c r="A25" t="s" s="2">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="E25" s="2"/>
       <c r="F25" t="s" s="2">
@@ -5685,14 +5691,14 @@
         <v>181</v>
       </c>
       <c r="L25" t="s" s="2">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="M25" t="s" s="2">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="N25" s="2"/>
       <c r="O25" t="s" s="2">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="P25" t="s" s="2">
         <v>88</v>
@@ -5717,13 +5723,13 @@
         <v>88</v>
       </c>
       <c r="X25" t="s" s="2">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="Y25" t="s" s="2">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="Z25" t="s" s="2">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="AA25" t="s" s="2">
         <v>88</v>
@@ -5741,7 +5747,7 @@
         <v>88</v>
       </c>
       <c r="AF25" t="s" s="2">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="AG25" t="s" s="2">
         <v>86</v>
@@ -5756,7 +5762,7 @@
         <v>88</v>
       </c>
       <c r="AK25" t="s" s="2">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="AL25" t="s" s="2">
         <v>88</v>
@@ -5768,7 +5774,7 @@
         <v>88</v>
       </c>
       <c r="AO25" t="s" s="2">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="AP25" t="s" s="2">
         <v>88</v>
@@ -5777,7 +5783,7 @@
         <v>88</v>
       </c>
       <c r="AR25" t="s" s="2">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="AS25" t="s" s="2">
         <v>88</v>
@@ -5786,21 +5792,21 @@
         <v>88</v>
       </c>
       <c r="AU25" t="s" s="2">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="AV25" t="s" s="2">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="AW25" t="s" s="2">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="26" hidden="true">
       <c r="A26" t="s" s="2">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
@@ -5936,10 +5942,10 @@
     </row>
     <row r="27" hidden="true">
       <c r="A27" t="s" s="2">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
@@ -6077,10 +6083,10 @@
     </row>
     <row r="28" hidden="true">
       <c r="A28" t="s" s="2">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -6103,19 +6109,19 @@
         <v>97</v>
       </c>
       <c r="K28" t="s" s="2">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="L28" t="s" s="2">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="M28" t="s" s="2">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="N28" t="s" s="2">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="O28" t="s" s="2">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="P28" t="s" s="2">
         <v>88</v>
@@ -6144,13 +6150,13 @@
       </c>
       <c r="Y28" s="2"/>
       <c r="Z28" t="s" s="2">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="AA28" t="s" s="2">
         <v>88</v>
       </c>
       <c r="AB28" t="s" s="2">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="AC28" s="2"/>
       <c r="AD28" t="s" s="2">
@@ -6160,7 +6166,7 @@
         <v>145</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>86</v>
@@ -6205,27 +6211,27 @@
         <v>88</v>
       </c>
       <c r="AU28" t="s" s="2">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="AV28" t="s" s="2">
         <v>88</v>
       </c>
       <c r="AW28" t="s" s="2">
-        <v>281</v>
+        <v>282</v>
       </c>
     </row>
     <row r="29" hidden="true">
       <c r="A29" t="s" s="2">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C29" t="s" s="2">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="D29" t="s" s="2">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="E29" s="2"/>
       <c r="F29" t="s" s="2">
@@ -6244,19 +6250,19 @@
         <v>97</v>
       </c>
       <c r="K29" t="s" s="2">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="L29" t="s" s="2">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="M29" t="s" s="2">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="N29" t="s" s="2">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="O29" t="s" s="2">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="P29" t="s" s="2">
         <v>88</v>
@@ -6281,13 +6287,13 @@
         <v>88</v>
       </c>
       <c r="X29" t="s" s="2">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="Y29" t="s" s="2">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="Z29" t="s" s="2">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="AA29" t="s" s="2">
         <v>88</v>
@@ -6305,7 +6311,7 @@
         <v>88</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="AG29" t="s" s="2">
         <v>86</v>
@@ -6350,21 +6356,21 @@
         <v>88</v>
       </c>
       <c r="AU29" t="s" s="2">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="AV29" t="s" s="2">
         <v>88</v>
       </c>
       <c r="AW29" t="s" s="2">
-        <v>281</v>
+        <v>282</v>
       </c>
     </row>
     <row r="30" hidden="true">
       <c r="A30" t="s" s="2">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
@@ -6500,10 +6506,10 @@
     </row>
     <row r="31" hidden="true">
       <c r="A31" t="s" s="2">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
@@ -6641,10 +6647,10 @@
     </row>
     <row r="32" hidden="true">
       <c r="A32" t="s" s="2">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
@@ -6670,23 +6676,23 @@
         <v>109</v>
       </c>
       <c r="L32" t="s" s="2">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="M32" t="s" s="2">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="N32" t="s" s="2">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="O32" t="s" s="2">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="P32" t="s" s="2">
         <v>88</v>
       </c>
       <c r="Q32" s="2"/>
       <c r="R32" t="s" s="2">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="S32" t="s" s="2">
         <v>88</v>
@@ -6728,7 +6734,7 @@
         <v>88</v>
       </c>
       <c r="AF32" t="s" s="2">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>86</v>
@@ -6773,21 +6779,21 @@
         <v>88</v>
       </c>
       <c r="AU32" t="s" s="2">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="AV32" t="s" s="2">
         <v>88</v>
       </c>
       <c r="AW32" t="s" s="2">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="33" hidden="true">
       <c r="A33" t="s" s="2">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
@@ -6813,13 +6819,13 @@
         <v>157</v>
       </c>
       <c r="L33" t="s" s="2">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="M33" t="s" s="2">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="N33" t="s" s="2">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="O33" s="2"/>
       <c r="P33" t="s" s="2">
@@ -6869,7 +6875,7 @@
         <v>88</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="AG33" t="s" s="2">
         <v>86</v>
@@ -6914,21 +6920,21 @@
         <v>88</v>
       </c>
       <c r="AU33" t="s" s="2">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="AV33" t="s" s="2">
         <v>88</v>
       </c>
       <c r="AW33" t="s" s="2">
-        <v>309</v>
+        <v>310</v>
       </c>
     </row>
     <row r="34" hidden="true">
       <c r="A34" t="s" s="2">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
@@ -6954,14 +6960,14 @@
         <v>115</v>
       </c>
       <c r="L34" t="s" s="2">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="M34" t="s" s="2">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="N34" s="2"/>
       <c r="O34" t="s" s="2">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="P34" t="s" s="2">
         <v>88</v>
@@ -7010,7 +7016,7 @@
         <v>88</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="AG34" t="s" s="2">
         <v>86</v>
@@ -7055,21 +7061,21 @@
         <v>88</v>
       </c>
       <c r="AU34" t="s" s="2">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="AV34" t="s" s="2">
         <v>88</v>
       </c>
       <c r="AW34" t="s" s="2">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="35" hidden="true">
       <c r="A35" t="s" s="2">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
@@ -7095,14 +7101,14 @@
         <v>157</v>
       </c>
       <c r="L35" t="s" s="2">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="M35" t="s" s="2">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="N35" s="2"/>
       <c r="O35" t="s" s="2">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="P35" t="s" s="2">
         <v>88</v>
@@ -7151,7 +7157,7 @@
         <v>88</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="AG35" t="s" s="2">
         <v>86</v>
@@ -7196,21 +7202,21 @@
         <v>88</v>
       </c>
       <c r="AU35" t="s" s="2">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="AV35" t="s" s="2">
         <v>88</v>
       </c>
       <c r="AW35" t="s" s="2">
-        <v>325</v>
+        <v>326</v>
       </c>
     </row>
     <row r="36" hidden="true">
       <c r="A36" t="s" s="2">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
@@ -7233,19 +7239,19 @@
         <v>97</v>
       </c>
       <c r="K36" t="s" s="2">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="L36" t="s" s="2">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="M36" t="s" s="2">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="N36" t="s" s="2">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="O36" t="s" s="2">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="P36" t="s" s="2">
         <v>88</v>
@@ -7294,7 +7300,7 @@
         <v>88</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>86</v>
@@ -7339,21 +7345,21 @@
         <v>88</v>
       </c>
       <c r="AU36" t="s" s="2">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="AV36" t="s" s="2">
         <v>88</v>
       </c>
       <c r="AW36" t="s" s="2">
-        <v>334</v>
+        <v>335</v>
       </c>
     </row>
     <row r="37" hidden="true">
       <c r="A37" t="s" s="2">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
@@ -7379,16 +7385,16 @@
         <v>157</v>
       </c>
       <c r="L37" t="s" s="2">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="M37" t="s" s="2">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="N37" t="s" s="2">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="O37" t="s" s="2">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="P37" t="s" s="2">
         <v>88</v>
@@ -7437,7 +7443,7 @@
         <v>88</v>
       </c>
       <c r="AF37" t="s" s="2">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="AG37" t="s" s="2">
         <v>86</v>
@@ -7482,25 +7488,25 @@
         <v>88</v>
       </c>
       <c r="AU37" t="s" s="2">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="AV37" t="s" s="2">
         <v>88</v>
       </c>
       <c r="AW37" t="s" s="2">
-        <v>342</v>
+        <v>343</v>
       </c>
     </row>
     <row r="38" hidden="true">
       <c r="A38" t="s" s="2">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E38" s="2"/>
       <c r="F38" t="s" s="2">
@@ -7519,13 +7525,13 @@
         <v>97</v>
       </c>
       <c r="K38" t="s" s="2">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="L38" t="s" s="2">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="M38" t="s" s="2">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="N38" s="2"/>
       <c r="O38" s="2"/>
@@ -7576,7 +7582,7 @@
         <v>88</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>96</v>
@@ -7600,7 +7606,7 @@
         <v>88</v>
       </c>
       <c r="AN38" t="s" s="2">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="AO38" t="s" s="2">
         <v>88</v>
@@ -7621,25 +7627,25 @@
         <v>88</v>
       </c>
       <c r="AU38" t="s" s="2">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="AV38" t="s" s="2">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="AW38" t="s" s="2">
-        <v>351</v>
+        <v>352</v>
       </c>
     </row>
     <row r="39" hidden="true">
       <c r="A39" t="s" s="2">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="E39" s="2"/>
       <c r="F39" t="s" s="2">
@@ -7658,13 +7664,13 @@
         <v>97</v>
       </c>
       <c r="K39" t="s" s="2">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="L39" t="s" s="2">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="M39" t="s" s="2">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="N39" s="2"/>
       <c r="O39" s="2"/>
@@ -7715,7 +7721,7 @@
         <v>88</v>
       </c>
       <c r="AF39" t="s" s="2">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="AG39" t="s" s="2">
         <v>86</v>
@@ -7760,21 +7766,21 @@
         <v>88</v>
       </c>
       <c r="AU39" t="s" s="2">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="AV39" t="s" s="2">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="AW39" t="s" s="2">
-        <v>359</v>
+        <v>360</v>
       </c>
     </row>
     <row r="40" hidden="true">
       <c r="A40" t="s" s="2">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
@@ -7797,13 +7803,13 @@
         <v>97</v>
       </c>
       <c r="K40" t="s" s="2">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="L40" t="s" s="2">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="M40" t="s" s="2">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="N40" s="2"/>
       <c r="O40" s="2"/>
@@ -7842,17 +7848,17 @@
         <v>88</v>
       </c>
       <c r="AB40" t="s" s="2">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="AC40" s="2"/>
       <c r="AD40" t="s" s="2">
         <v>88</v>
       </c>
       <c r="AE40" t="s" s="2">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="AF40" t="s" s="2">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="AG40" t="s" s="2">
         <v>86</v>
@@ -7876,7 +7882,7 @@
         <v>88</v>
       </c>
       <c r="AN40" t="s" s="2">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="AO40" t="s" s="2">
         <v>88</v>
@@ -7897,24 +7903,24 @@
         <v>88</v>
       </c>
       <c r="AU40" t="s" s="2">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="AV40" t="s" s="2">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="AW40" t="s" s="2">
-        <v>369</v>
+        <v>370</v>
       </c>
     </row>
     <row r="41" hidden="true">
       <c r="A41" t="s" s="2">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="C41" t="s" s="2">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="D41" t="s" s="2">
         <v>88</v>
@@ -7936,13 +7942,13 @@
         <v>97</v>
       </c>
       <c r="K41" t="s" s="2">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="L41" t="s" s="2">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="M41" t="s" s="2">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="N41" s="2"/>
       <c r="O41" s="2"/>
@@ -7993,7 +7999,7 @@
         <v>88</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="AG41" t="s" s="2">
         <v>86</v>
@@ -8038,21 +8044,21 @@
         <v>88</v>
       </c>
       <c r="AU41" t="s" s="2">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="AV41" t="s" s="2">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="AW41" t="s" s="2">
-        <v>369</v>
+        <v>370</v>
       </c>
     </row>
     <row r="42" hidden="true">
       <c r="A42" t="s" s="2">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
@@ -8188,10 +8194,10 @@
     </row>
     <row r="43" hidden="true">
       <c r="A43" t="s" s="2">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
@@ -8329,14 +8335,14 @@
     </row>
     <row r="44" hidden="true">
       <c r="A44" t="s" s="2">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="E44" s="2"/>
       <c r="F44" t="s" s="2">
@@ -8355,16 +8361,16 @@
         <v>97</v>
       </c>
       <c r="K44" t="s" s="2">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="L44" t="s" s="2">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="M44" t="s" s="2">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="N44" t="s" s="2">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="O44" s="2"/>
       <c r="P44" t="s" s="2">
@@ -8414,7 +8420,7 @@
         <v>88</v>
       </c>
       <c r="AF44" t="s" s="2">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="AG44" t="s" s="2">
         <v>86</v>
@@ -8423,13 +8429,13 @@
         <v>96</v>
       </c>
       <c r="AI44" t="s" s="2">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="AJ44" t="s" s="2">
         <v>88</v>
       </c>
       <c r="AK44" t="s" s="2">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="AL44" t="s" s="2">
         <v>88</v>
@@ -8441,7 +8447,7 @@
         <v>88</v>
       </c>
       <c r="AO44" t="s" s="2">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="AP44" t="s" s="2">
         <v>88</v>
@@ -8450,7 +8456,7 @@
         <v>88</v>
       </c>
       <c r="AR44" t="s" s="2">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="AS44" t="s" s="2">
         <v>88</v>
@@ -8459,25 +8465,25 @@
         <v>88</v>
       </c>
       <c r="AU44" t="s" s="2">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="AV44" t="s" s="2">
         <v>88</v>
       </c>
       <c r="AW44" t="s" s="2">
-        <v>387</v>
+        <v>388</v>
       </c>
     </row>
     <row r="45" hidden="true">
       <c r="A45" t="s" s="2">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="E45" s="2"/>
       <c r="F45" t="s" s="2">
@@ -8496,23 +8502,23 @@
         <v>97</v>
       </c>
       <c r="K45" t="s" s="2">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="L45" t="s" s="2">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="M45" t="s" s="2">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="N45" t="s" s="2">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="O45" s="2"/>
       <c r="P45" t="s" s="2">
         <v>88</v>
       </c>
       <c r="Q45" t="s" s="2">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="R45" t="s" s="2">
         <v>88</v>
@@ -8557,7 +8563,7 @@
         <v>88</v>
       </c>
       <c r="AF45" t="s" s="2">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="AG45" t="s" s="2">
         <v>86</v>
@@ -8566,13 +8572,13 @@
         <v>96</v>
       </c>
       <c r="AI45" t="s" s="2">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="AJ45" t="s" s="2">
         <v>88</v>
       </c>
       <c r="AK45" t="s" s="2">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="AL45" t="s" s="2">
         <v>88</v>
@@ -8584,7 +8590,7 @@
         <v>88</v>
       </c>
       <c r="AO45" t="s" s="2">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="AP45" t="s" s="2">
         <v>88</v>
@@ -8593,7 +8599,7 @@
         <v>88</v>
       </c>
       <c r="AR45" t="s" s="2">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="AS45" t="s" s="2">
         <v>88</v>
@@ -8602,25 +8608,25 @@
         <v>88</v>
       </c>
       <c r="AU45" t="s" s="2">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="AV45" t="s" s="2">
         <v>88</v>
       </c>
       <c r="AW45" t="s" s="2">
-        <v>398</v>
+        <v>399</v>
       </c>
     </row>
     <row r="46" hidden="true">
       <c r="A46" t="s" s="2">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="E46" s="2"/>
       <c r="F46" t="s" s="2">
@@ -8639,16 +8645,16 @@
         <v>97</v>
       </c>
       <c r="K46" t="s" s="2">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="L46" t="s" s="2">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="M46" t="s" s="2">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="N46" t="s" s="2">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="O46" s="2"/>
       <c r="P46" t="s" s="2">
@@ -8698,7 +8704,7 @@
         <v>88</v>
       </c>
       <c r="AF46" t="s" s="2">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="AG46" t="s" s="2">
         <v>86</v>
@@ -8710,10 +8716,10 @@
         <v>88</v>
       </c>
       <c r="AJ46" t="s" s="2">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="AK46" t="s" s="2">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="AL46" t="s" s="2">
         <v>88</v>
@@ -8725,7 +8731,7 @@
         <v>88</v>
       </c>
       <c r="AO46" t="s" s="2">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="AP46" t="s" s="2">
         <v>88</v>
@@ -8734,7 +8740,7 @@
         <v>88</v>
       </c>
       <c r="AR46" t="s" s="2">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="AS46" t="s" s="2">
         <v>88</v>
@@ -8743,7 +8749,7 @@
         <v>88</v>
       </c>
       <c r="AU46" t="s" s="2">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AV46" t="s" s="2">
         <v>88</v>
@@ -8754,10 +8760,10 @@
     </row>
     <row r="47" hidden="true">
       <c r="A47" t="s" s="2">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" t="s" s="2">
@@ -8893,10 +8899,10 @@
     </row>
     <row r="48" hidden="true">
       <c r="A48" t="s" s="2">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" t="s" s="2">
@@ -9034,14 +9040,14 @@
     </row>
     <row r="49" hidden="true">
       <c r="A49" t="s" s="2">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="B49" t="s" s="2">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" t="s" s="2">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="E49" s="2"/>
       <c r="F49" t="s" s="2">
@@ -9063,10 +9069,10 @@
         <v>141</v>
       </c>
       <c r="L49" t="s" s="2">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="M49" t="s" s="2">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="N49" t="s" s="2">
         <v>167</v>
@@ -9119,7 +9125,7 @@
         <v>88</v>
       </c>
       <c r="AF49" t="s" s="2">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="AG49" t="s" s="2">
         <v>86</v>
@@ -9175,10 +9181,10 @@
     </row>
     <row r="50" hidden="true">
       <c r="A50" t="s" s="2">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="B50" t="s" s="2">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="C50" s="2"/>
       <c r="D50" t="s" s="2">
@@ -9204,10 +9210,10 @@
         <v>181</v>
       </c>
       <c r="L50" t="s" s="2">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="M50" t="s" s="2">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="N50" s="2"/>
       <c r="O50" s="2"/>
@@ -9234,13 +9240,13 @@
         <v>88</v>
       </c>
       <c r="X50" t="s" s="2">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="Y50" t="s" s="2">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="Z50" t="s" s="2">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="AA50" t="s" s="2">
         <v>88</v>
@@ -9258,7 +9264,7 @@
         <v>88</v>
       </c>
       <c r="AF50" t="s" s="2">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="AG50" t="s" s="2">
         <v>86</v>
@@ -9303,21 +9309,21 @@
         <v>88</v>
       </c>
       <c r="AU50" t="s" s="2">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="AV50" t="s" s="2">
         <v>88</v>
       </c>
       <c r="AW50" t="s" s="2">
-        <v>420</v>
+        <v>421</v>
       </c>
     </row>
     <row r="51" hidden="true">
       <c r="A51" t="s" s="2">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="B51" t="s" s="2">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="C51" s="2"/>
       <c r="D51" t="s" s="2">
@@ -9453,10 +9459,10 @@
     </row>
     <row r="52" hidden="true">
       <c r="A52" t="s" s="2">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="B52" t="s" s="2">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="C52" s="2"/>
       <c r="D52" t="s" s="2">
@@ -9594,10 +9600,10 @@
     </row>
     <row r="53" hidden="true">
       <c r="A53" t="s" s="2">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="B53" t="s" s="2">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" t="s" s="2">
@@ -9620,19 +9626,19 @@
         <v>97</v>
       </c>
       <c r="K53" t="s" s="2">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="L53" t="s" s="2">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="M53" t="s" s="2">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="N53" t="s" s="2">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="O53" t="s" s="2">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="P53" t="s" s="2">
         <v>88</v>
@@ -9669,7 +9675,7 @@
         <v>88</v>
       </c>
       <c r="AB53" t="s" s="2">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="AC53" s="2"/>
       <c r="AD53" t="s" s="2">
@@ -9679,7 +9685,7 @@
         <v>145</v>
       </c>
       <c r="AF53" t="s" s="2">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="AG53" t="s" s="2">
         <v>86</v>
@@ -9724,27 +9730,27 @@
         <v>88</v>
       </c>
       <c r="AU53" t="s" s="2">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="AV53" t="s" s="2">
         <v>88</v>
       </c>
       <c r="AW53" t="s" s="2">
-        <v>281</v>
+        <v>282</v>
       </c>
     </row>
     <row r="54" hidden="true">
       <c r="A54" t="s" s="2">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="B54" t="s" s="2">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="C54" t="s" s="2">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="D54" t="s" s="2">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="E54" s="2"/>
       <c r="F54" t="s" s="2">
@@ -9763,19 +9769,19 @@
         <v>97</v>
       </c>
       <c r="K54" t="s" s="2">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="L54" t="s" s="2">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="M54" t="s" s="2">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="N54" t="s" s="2">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="O54" t="s" s="2">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="P54" t="s" s="2">
         <v>88</v>
@@ -9800,11 +9806,11 @@
         <v>88</v>
       </c>
       <c r="X54" t="s" s="2">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="Y54" s="2"/>
       <c r="Z54" t="s" s="2">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="AA54" t="s" s="2">
         <v>88</v>
@@ -9822,7 +9828,7 @@
         <v>88</v>
       </c>
       <c r="AF54" t="s" s="2">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="AG54" t="s" s="2">
         <v>86</v>
@@ -9843,7 +9849,7 @@
         <v>88</v>
       </c>
       <c r="AM54" t="s" s="2">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="AN54" t="s" s="2">
         <v>88</v>
@@ -9855,7 +9861,7 @@
         <v>88</v>
       </c>
       <c r="AQ54" t="s" s="2">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="AR54" t="s" s="2">
         <v>88</v>
@@ -9864,24 +9870,24 @@
         <v>88</v>
       </c>
       <c r="AT54" t="s" s="2">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="AU54" t="s" s="2">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="AV54" t="s" s="2">
         <v>88</v>
       </c>
       <c r="AW54" t="s" s="2">
-        <v>281</v>
+        <v>282</v>
       </c>
     </row>
     <row r="55" hidden="true">
       <c r="A55" t="s" s="2">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="B55" t="s" s="2">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="C55" s="2"/>
       <c r="D55" t="s" s="2">
@@ -9907,16 +9913,16 @@
         <v>157</v>
       </c>
       <c r="L55" t="s" s="2">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="M55" t="s" s="2">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="N55" t="s" s="2">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="O55" t="s" s="2">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="P55" t="s" s="2">
         <v>88</v>
@@ -9965,7 +9971,7 @@
         <v>88</v>
       </c>
       <c r="AF55" t="s" s="2">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="AG55" t="s" s="2">
         <v>86</v>
@@ -10010,21 +10016,21 @@
         <v>88</v>
       </c>
       <c r="AU55" t="s" s="2">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="AV55" t="s" s="2">
         <v>88</v>
       </c>
       <c r="AW55" t="s" s="2">
-        <v>342</v>
+        <v>343</v>
       </c>
     </row>
     <row r="56" hidden="true">
       <c r="A56" t="s" s="2">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="B56" t="s" s="2">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="C56" s="2"/>
       <c r="D56" t="s" s="2">
@@ -10047,17 +10053,17 @@
         <v>97</v>
       </c>
       <c r="K56" t="s" s="2">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="L56" t="s" s="2">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="M56" t="s" s="2">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="N56" s="2"/>
       <c r="O56" t="s" s="2">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="P56" t="s" s="2">
         <v>88</v>
@@ -10106,7 +10112,7 @@
         <v>88</v>
       </c>
       <c r="AF56" t="s" s="2">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="AG56" t="s" s="2">
         <v>96</v>
@@ -10151,21 +10157,21 @@
         <v>88</v>
       </c>
       <c r="AU56" t="s" s="2">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="AV56" t="s" s="2">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="AW56" t="s" s="2">
-        <v>440</v>
+        <v>441</v>
       </c>
     </row>
     <row r="57" hidden="true">
       <c r="A57" t="s" s="2">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="B57" t="s" s="2">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="C57" s="2"/>
       <c r="D57" t="s" s="2">
@@ -10301,14 +10307,14 @@
     </row>
     <row r="58" hidden="true">
       <c r="A58" t="s" s="2">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="B58" t="s" s="2">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="C58" s="2"/>
       <c r="D58" t="s" s="2">
-        <v>88</v>
+        <v>164</v>
       </c>
       <c r="E58" s="2"/>
       <c r="F58" t="s" s="2">
@@ -10330,12 +10336,14 @@
         <v>141</v>
       </c>
       <c r="L58" t="s" s="2">
-        <v>142</v>
+        <v>165</v>
       </c>
       <c r="M58" t="s" s="2">
-        <v>143</v>
-      </c>
-      <c r="N58" s="2"/>
+        <v>166</v>
+      </c>
+      <c r="N58" t="s" s="2">
+        <v>167</v>
+      </c>
       <c r="O58" s="2"/>
       <c r="P58" t="s" s="2">
         <v>88</v>
@@ -10429,7 +10437,7 @@
         <v>88</v>
       </c>
       <c r="AU58" t="s" s="2">
-        <v>88</v>
+        <v>161</v>
       </c>
       <c r="AV58" t="s" s="2">
         <v>88</v>
@@ -10440,13 +10448,13 @@
     </row>
     <row r="59" hidden="true">
       <c r="A59" t="s" s="2">
+        <v>444</v>
+      </c>
+      <c r="B59" t="s" s="2">
         <v>443</v>
       </c>
-      <c r="B59" t="s" s="2">
-        <v>442</v>
-      </c>
       <c r="C59" t="s" s="2">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="D59" t="s" s="2">
         <v>88</v>
@@ -10468,13 +10476,13 @@
         <v>88</v>
       </c>
       <c r="K59" t="s" s="2">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="L59" t="s" s="2">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="M59" t="s" s="2">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="N59" s="2"/>
       <c r="O59" s="2"/>
@@ -10581,10 +10589,10 @@
     </row>
     <row r="60" hidden="true">
       <c r="A60" t="s" s="2">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="B60" t="s" s="2">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="C60" s="2"/>
       <c r="D60" t="s" s="2">
@@ -10610,13 +10618,13 @@
         <v>157</v>
       </c>
       <c r="L60" t="s" s="2">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="M60" t="s" s="2">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="N60" t="s" s="2">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="O60" s="2"/>
       <c r="P60" t="s" s="2">
@@ -10666,7 +10674,7 @@
         <v>88</v>
       </c>
       <c r="AF60" t="s" s="2">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="AG60" t="s" s="2">
         <v>86</v>
@@ -10675,7 +10683,7 @@
         <v>96</v>
       </c>
       <c r="AI60" t="s" s="2">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="AJ60" t="s" s="2">
         <v>88</v>
@@ -10722,10 +10730,10 @@
     </row>
     <row r="61" hidden="true">
       <c r="A61" t="s" s="2">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="B61" t="s" s="2">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="C61" s="2"/>
       <c r="D61" t="s" s="2">
@@ -10748,16 +10756,16 @@
         <v>97</v>
       </c>
       <c r="K61" t="s" s="2">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="L61" t="s" s="2">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="M61" t="s" s="2">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="N61" t="s" s="2">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="O61" s="2"/>
       <c r="P61" t="s" s="2">
@@ -10807,7 +10815,7 @@
         <v>88</v>
       </c>
       <c r="AF61" t="s" s="2">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="AG61" t="s" s="2">
         <v>86</v>
@@ -10852,7 +10860,7 @@
         <v>88</v>
       </c>
       <c r="AU61" t="s" s="2">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="AV61" t="s" s="2">
         <v>88</v>
@@ -10863,10 +10871,10 @@
     </row>
     <row r="62" hidden="true">
       <c r="A62" t="s" s="2">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="B62" t="s" s="2">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="C62" s="2"/>
       <c r="D62" t="s" s="2">
@@ -10892,13 +10900,13 @@
         <v>157</v>
       </c>
       <c r="L62" t="s" s="2">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="M62" t="s" s="2">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="N62" t="s" s="2">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="O62" s="2"/>
       <c r="P62" t="s" s="2">
@@ -10948,7 +10956,7 @@
         <v>88</v>
       </c>
       <c r="AF62" t="s" s="2">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="AG62" t="s" s="2">
         <v>86</v>
@@ -11004,10 +11012,10 @@
     </row>
     <row r="63" hidden="true">
       <c r="A63" t="s" s="2">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="B63" t="s" s="2">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="C63" s="2"/>
       <c r="D63" t="s" s="2">
@@ -11030,17 +11038,17 @@
         <v>88</v>
       </c>
       <c r="K63" t="s" s="2">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="L63" t="s" s="2">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="M63" t="s" s="2">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="N63" s="2"/>
       <c r="O63" t="s" s="2">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="P63" t="s" s="2">
         <v>88</v>
@@ -11089,7 +11097,7 @@
         <v>88</v>
       </c>
       <c r="AF63" t="s" s="2">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="AG63" t="s" s="2">
         <v>86</v>
@@ -11134,7 +11142,7 @@
         <v>88</v>
       </c>
       <c r="AU63" t="s" s="2">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="AV63" t="s" s="2">
         <v>88</v>
@@ -11145,10 +11153,10 @@
     </row>
     <row r="64" hidden="true">
       <c r="A64" t="s" s="2">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="B64" t="s" s="2">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="C64" s="2"/>
       <c r="D64" t="s" s="2">
@@ -11171,17 +11179,17 @@
         <v>97</v>
       </c>
       <c r="K64" t="s" s="2">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="L64" t="s" s="2">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="M64" t="s" s="2">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="N64" s="2"/>
       <c r="O64" t="s" s="2">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="P64" t="s" s="2">
         <v>88</v>
@@ -11230,7 +11238,7 @@
         <v>88</v>
       </c>
       <c r="AF64" t="s" s="2">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="AG64" t="s" s="2">
         <v>86</v>
@@ -11275,10 +11283,10 @@
         <v>88</v>
       </c>
       <c r="AU64" t="s" s="2">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="AV64" t="s" s="2">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="AW64" t="s" s="2">
         <v>88</v>
@@ -11286,10 +11294,10 @@
     </row>
     <row r="65" hidden="true">
       <c r="A65" t="s" s="2">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="B65" t="s" s="2">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="C65" s="2"/>
       <c r="D65" t="s" s="2">
@@ -11425,10 +11433,10 @@
     </row>
     <row r="66" hidden="true">
       <c r="A66" t="s" s="2">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="B66" t="s" s="2">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="C66" s="2"/>
       <c r="D66" t="s" s="2">
@@ -11566,10 +11574,10 @@
     </row>
     <row r="67" hidden="true">
       <c r="A67" t="s" s="2">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="B67" t="s" s="2">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="C67" s="2"/>
       <c r="D67" t="s" s="2">
@@ -11595,13 +11603,13 @@
         <v>157</v>
       </c>
       <c r="L67" t="s" s="2">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="M67" t="s" s="2">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="N67" t="s" s="2">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="O67" s="2"/>
       <c r="P67" t="s" s="2">
@@ -11651,7 +11659,7 @@
         <v>88</v>
       </c>
       <c r="AF67" t="s" s="2">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="AG67" t="s" s="2">
         <v>86</v>
@@ -11660,7 +11668,7 @@
         <v>96</v>
       </c>
       <c r="AI67" t="s" s="2">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="AJ67" t="s" s="2">
         <v>88</v>
@@ -11707,10 +11715,10 @@
     </row>
     <row r="68" hidden="true">
       <c r="A68" t="s" s="2">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="B68" t="s" s="2">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="C68" s="2"/>
       <c r="D68" t="s" s="2">
@@ -11733,16 +11741,16 @@
         <v>97</v>
       </c>
       <c r="K68" t="s" s="2">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="L68" t="s" s="2">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="M68" t="s" s="2">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="N68" t="s" s="2">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="O68" s="2"/>
       <c r="P68" t="s" s="2">
@@ -11792,7 +11800,7 @@
         <v>88</v>
       </c>
       <c r="AF68" t="s" s="2">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="AG68" t="s" s="2">
         <v>86</v>
@@ -11837,7 +11845,7 @@
         <v>88</v>
       </c>
       <c r="AU68" t="s" s="2">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="AV68" t="s" s="2">
         <v>88</v>
@@ -11848,10 +11856,10 @@
     </row>
     <row r="69" hidden="true">
       <c r="A69" t="s" s="2">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="B69" t="s" s="2">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="C69" s="2"/>
       <c r="D69" t="s" s="2">
@@ -11877,13 +11885,13 @@
         <v>157</v>
       </c>
       <c r="L69" t="s" s="2">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="M69" t="s" s="2">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="N69" t="s" s="2">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="O69" s="2"/>
       <c r="P69" t="s" s="2">
@@ -11933,7 +11941,7 @@
         <v>88</v>
       </c>
       <c r="AF69" t="s" s="2">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="AG69" t="s" s="2">
         <v>86</v>
@@ -11989,10 +11997,10 @@
     </row>
     <row r="70" hidden="true">
       <c r="A70" t="s" s="2">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="B70" t="s" s="2">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="C70" s="2"/>
       <c r="D70" t="s" s="2">
@@ -12018,10 +12026,10 @@
         <v>181</v>
       </c>
       <c r="L70" t="s" s="2">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="M70" t="s" s="2">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="N70" s="2"/>
       <c r="O70" s="2"/>
@@ -12048,13 +12056,13 @@
         <v>88</v>
       </c>
       <c r="X70" t="s" s="2">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="Y70" t="s" s="2">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="Z70" t="s" s="2">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="AA70" t="s" s="2">
         <v>88</v>
@@ -12072,7 +12080,7 @@
         <v>88</v>
       </c>
       <c r="AF70" t="s" s="2">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="AG70" t="s" s="2">
         <v>86</v>
@@ -12117,10 +12125,10 @@
         <v>88</v>
       </c>
       <c r="AU70" t="s" s="2">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="AV70" t="s" s="2">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="AW70" t="s" s="2">
         <v>88</v>
@@ -12128,14 +12136,14 @@
     </row>
     <row r="71" hidden="true">
       <c r="A71" t="s" s="2">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="B71" t="s" s="2">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="C71" s="2"/>
       <c r="D71" t="s" s="2">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="E71" s="2"/>
       <c r="F71" t="s" s="2">
@@ -12154,16 +12162,16 @@
         <v>97</v>
       </c>
       <c r="K71" t="s" s="2">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="L71" t="s" s="2">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="M71" t="s" s="2">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="N71" t="s" s="2">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="O71" s="2"/>
       <c r="P71" t="s" s="2">
@@ -12213,7 +12221,7 @@
         <v>88</v>
       </c>
       <c r="AF71" t="s" s="2">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="AG71" t="s" s="2">
         <v>86</v>
@@ -12228,7 +12236,7 @@
         <v>88</v>
       </c>
       <c r="AK71" t="s" s="2">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="AL71" t="s" s="2">
         <v>88</v>
@@ -12240,7 +12248,7 @@
         <v>88</v>
       </c>
       <c r="AO71" t="s" s="2">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="AP71" t="s" s="2">
         <v>88</v>
@@ -12249,7 +12257,7 @@
         <v>88</v>
       </c>
       <c r="AR71" t="s" s="2">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="AS71" t="s" s="2">
         <v>88</v>
@@ -12258,10 +12266,10 @@
         <v>88</v>
       </c>
       <c r="AU71" t="s" s="2">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="AV71" t="s" s="2">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="AW71" t="s" s="2">
         <v>88</v>
@@ -12269,14 +12277,14 @@
     </row>
     <row r="72" hidden="true">
       <c r="A72" t="s" s="2">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="B72" t="s" s="2">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="C72" s="2"/>
       <c r="D72" t="s" s="2">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="E72" s="2"/>
       <c r="F72" t="s" s="2">
@@ -12298,10 +12306,10 @@
         <v>181</v>
       </c>
       <c r="L72" t="s" s="2">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="M72" t="s" s="2">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="N72" s="2"/>
       <c r="O72" s="2"/>
@@ -12331,10 +12339,10 @@
         <v>119</v>
       </c>
       <c r="Y72" t="s" s="2">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="Z72" t="s" s="2">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="AA72" t="s" s="2">
         <v>88</v>
@@ -12352,7 +12360,7 @@
         <v>88</v>
       </c>
       <c r="AF72" t="s" s="2">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="AG72" t="s" s="2">
         <v>86</v>
@@ -12367,7 +12375,7 @@
         <v>88</v>
       </c>
       <c r="AK72" t="s" s="2">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="AL72" t="s" s="2">
         <v>88</v>
@@ -12379,7 +12387,7 @@
         <v>88</v>
       </c>
       <c r="AO72" t="s" s="2">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="AP72" t="s" s="2">
         <v>88</v>
@@ -12388,7 +12396,7 @@
         <v>88</v>
       </c>
       <c r="AR72" t="s" s="2">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="AS72" t="s" s="2">
         <v>88</v>
@@ -12397,21 +12405,21 @@
         <v>88</v>
       </c>
       <c r="AU72" t="s" s="2">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="AV72" t="s" s="2">
         <v>88</v>
       </c>
       <c r="AW72" t="s" s="2">
-        <v>504</v>
+        <v>505</v>
       </c>
     </row>
     <row r="73" hidden="true">
       <c r="A73" t="s" s="2">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="B73" t="s" s="2">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="C73" s="2"/>
       <c r="D73" t="s" s="2">
@@ -12547,10 +12555,10 @@
     </row>
     <row r="74" hidden="true">
       <c r="A74" t="s" s="2">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="B74" t="s" s="2">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="C74" s="2"/>
       <c r="D74" t="s" s="2">
@@ -12686,13 +12694,13 @@
     </row>
     <row r="75" hidden="true">
       <c r="A75" t="s" s="2">
+        <v>508</v>
+      </c>
+      <c r="B75" t="s" s="2">
         <v>507</v>
       </c>
-      <c r="B75" t="s" s="2">
-        <v>506</v>
-      </c>
       <c r="C75" t="s" s="2">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="D75" t="s" s="2">
         <v>88</v>
@@ -12714,13 +12722,13 @@
         <v>88</v>
       </c>
       <c r="K75" t="s" s="2">
+        <v>510</v>
+      </c>
+      <c r="L75" t="s" s="2">
         <v>509</v>
       </c>
-      <c r="L75" t="s" s="2">
-        <v>508</v>
-      </c>
       <c r="M75" t="s" s="2">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="N75" s="2"/>
       <c r="O75" s="2"/>
@@ -12827,10 +12835,10 @@
     </row>
     <row r="76" hidden="true">
       <c r="A76" t="s" s="2">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="B76" t="s" s="2">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="C76" s="2"/>
       <c r="D76" t="s" s="2">
@@ -12966,10 +12974,10 @@
     </row>
     <row r="77" hidden="true">
       <c r="A77" t="s" s="2">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="B77" t="s" s="2">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="C77" s="2"/>
       <c r="D77" t="s" s="2">
@@ -13107,10 +13115,10 @@
     </row>
     <row r="78" hidden="true">
       <c r="A78" t="s" s="2">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="B78" t="s" s="2">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="C78" s="2"/>
       <c r="D78" t="s" s="2">
@@ -13150,7 +13158,7 @@
       </c>
       <c r="Q78" s="2"/>
       <c r="R78" t="s" s="2">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="S78" t="s" s="2">
         <v>88</v>
@@ -13248,10 +13256,10 @@
     </row>
     <row r="79" hidden="true">
       <c r="A79" t="s" s="2">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="B79" t="s" s="2">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="C79" s="2"/>
       <c r="D79" t="s" s="2">
@@ -13277,10 +13285,10 @@
         <v>181</v>
       </c>
       <c r="L79" t="s" s="2">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="M79" t="s" s="2">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="N79" s="2"/>
       <c r="O79" s="2"/>
@@ -13319,17 +13327,17 @@
         <v>88</v>
       </c>
       <c r="AB79" t="s" s="2">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="AC79" s="2"/>
       <c r="AD79" t="s" s="2">
         <v>88</v>
       </c>
       <c r="AE79" t="s" s="2">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="AF79" t="s" s="2">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="AG79" t="s" s="2">
         <v>86</v>
@@ -13385,10 +13393,10 @@
     </row>
     <row r="80" hidden="true">
       <c r="A80" t="s" s="2">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="B80" t="s" s="2">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="C80" t="s" s="2">
         <v>179</v>
@@ -13416,10 +13424,10 @@
         <v>181</v>
       </c>
       <c r="L80" t="s" s="2">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="M80" t="s" s="2">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="N80" s="2"/>
       <c r="O80" s="2"/>
@@ -13449,10 +13457,10 @@
         <v>119</v>
       </c>
       <c r="Y80" t="s" s="2">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="Z80" t="s" s="2">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="AA80" t="s" s="2">
         <v>88</v>
@@ -13470,7 +13478,7 @@
         <v>88</v>
       </c>
       <c r="AF80" t="s" s="2">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="AG80" t="s" s="2">
         <v>86</v>
@@ -13485,7 +13493,7 @@
         <v>88</v>
       </c>
       <c r="AK80" t="s" s="2">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="AL80" t="s" s="2">
         <v>88</v>
@@ -13526,10 +13534,10 @@
     </row>
     <row r="81" hidden="true">
       <c r="A81" t="s" s="2">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="B81" t="s" s="2">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="C81" s="2"/>
       <c r="D81" t="s" s="2">
@@ -13552,19 +13560,19 @@
         <v>97</v>
       </c>
       <c r="K81" t="s" s="2">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="L81" t="s" s="2">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="M81" t="s" s="2">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="N81" t="s" s="2">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="O81" t="s" s="2">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="P81" t="s" s="2">
         <v>88</v>
@@ -13613,7 +13621,7 @@
         <v>88</v>
       </c>
       <c r="AF81" t="s" s="2">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="AG81" t="s" s="2">
         <v>86</v>
@@ -13658,21 +13666,21 @@
         <v>88</v>
       </c>
       <c r="AU81" t="s" s="2">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="AV81" t="s" s="2">
         <v>88</v>
       </c>
       <c r="AW81" t="s" s="2">
-        <v>281</v>
+        <v>282</v>
       </c>
     </row>
     <row r="82" hidden="true">
       <c r="A82" t="s" s="2">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="B82" t="s" s="2">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="C82" s="2"/>
       <c r="D82" t="s" s="2">
@@ -13698,16 +13706,16 @@
         <v>157</v>
       </c>
       <c r="L82" t="s" s="2">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="M82" t="s" s="2">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="N82" t="s" s="2">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="O82" t="s" s="2">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="P82" t="s" s="2">
         <v>88</v>
@@ -13756,7 +13764,7 @@
         <v>88</v>
       </c>
       <c r="AF82" t="s" s="2">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="AG82" t="s" s="2">
         <v>86</v>
@@ -13801,21 +13809,21 @@
         <v>88</v>
       </c>
       <c r="AU82" t="s" s="2">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="AV82" t="s" s="2">
         <v>88</v>
       </c>
       <c r="AW82" t="s" s="2">
-        <v>342</v>
+        <v>343</v>
       </c>
     </row>
     <row r="83" hidden="true">
       <c r="A83" t="s" s="2">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="B83" t="s" s="2">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="C83" s="2"/>
       <c r="D83" t="s" s="2">
@@ -13841,13 +13849,13 @@
         <v>181</v>
       </c>
       <c r="L83" t="s" s="2">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="M83" t="s" s="2">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="N83" t="s" s="2">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="O83" s="2"/>
       <c r="P83" t="s" s="2">
@@ -13873,13 +13881,13 @@
         <v>88</v>
       </c>
       <c r="X83" t="s" s="2">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="Y83" t="s" s="2">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="Z83" t="s" s="2">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="AA83" t="s" s="2">
         <v>88</v>
@@ -13897,7 +13905,7 @@
         <v>88</v>
       </c>
       <c r="AF83" t="s" s="2">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="AG83" t="s" s="2">
         <v>86</v>
@@ -13942,7 +13950,7 @@
         <v>88</v>
       </c>
       <c r="AU83" t="s" s="2">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="AV83" t="s" s="2">
         <v>88</v>
@@ -13953,10 +13961,10 @@
     </row>
     <row r="84" hidden="true">
       <c r="A84" t="s" s="2">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="B84" t="s" s="2">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="C84" s="2"/>
       <c r="D84" t="s" s="2">
@@ -13979,16 +13987,16 @@
         <v>88</v>
       </c>
       <c r="K84" t="s" s="2">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="L84" t="s" s="2">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="M84" t="s" s="2">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="N84" t="s" s="2">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="O84" s="2"/>
       <c r="P84" t="s" s="2">
@@ -14038,7 +14046,7 @@
         <v>88</v>
       </c>
       <c r="AF84" t="s" s="2">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="AG84" t="s" s="2">
         <v>86</v>
@@ -14056,7 +14064,7 @@
         <v>88</v>
       </c>
       <c r="AL84" t="s" s="2">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="AM84" t="s" s="2">
         <v>88</v>
@@ -14068,7 +14076,7 @@
         <v>88</v>
       </c>
       <c r="AP84" t="s" s="2">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="AQ84" t="s" s="2">
         <v>88</v>
@@ -14077,13 +14085,13 @@
         <v>88</v>
       </c>
       <c r="AS84" t="s" s="2">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="AT84" t="s" s="2">
         <v>88</v>
       </c>
       <c r="AU84" t="s" s="2">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="AV84" t="s" s="2">
         <v>88</v>
@@ -14094,10 +14102,10 @@
     </row>
     <row r="85" hidden="true">
       <c r="A85" t="s" s="2">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="B85" t="s" s="2">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="C85" s="2"/>
       <c r="D85" t="s" s="2">
@@ -14123,13 +14131,13 @@
         <v>181</v>
       </c>
       <c r="L85" t="s" s="2">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="M85" t="s" s="2">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="N85" t="s" s="2">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="O85" s="2"/>
       <c r="P85" t="s" s="2">
@@ -14155,13 +14163,13 @@
         <v>88</v>
       </c>
       <c r="X85" t="s" s="2">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="Y85" t="s" s="2">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="Z85" t="s" s="2">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="AA85" t="s" s="2">
         <v>88</v>
@@ -14179,7 +14187,7 @@
         <v>88</v>
       </c>
       <c r="AF85" t="s" s="2">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="AG85" t="s" s="2">
         <v>86</v>
@@ -14224,7 +14232,7 @@
         <v>88</v>
       </c>
       <c r="AU85" t="s" s="2">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="AV85" t="s" s="2">
         <v>88</v>
@@ -14235,10 +14243,10 @@
     </row>
     <row r="86" hidden="true">
       <c r="A86" t="s" s="2">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="B86" t="s" s="2">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="C86" s="2"/>
       <c r="D86" t="s" s="2">
@@ -14261,17 +14269,17 @@
         <v>88</v>
       </c>
       <c r="K86" t="s" s="2">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="L86" t="s" s="2">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="M86" t="s" s="2">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="N86" s="2"/>
       <c r="O86" t="s" s="2">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="P86" t="s" s="2">
         <v>88</v>
@@ -14320,7 +14328,7 @@
         <v>88</v>
       </c>
       <c r="AF86" t="s" s="2">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="AG86" t="s" s="2">
         <v>86</v>
@@ -14365,7 +14373,7 @@
         <v>88</v>
       </c>
       <c r="AU86" t="s" s="2">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="AV86" t="s" s="2">
         <v>88</v>
@@ -14376,10 +14384,10 @@
     </row>
     <row r="87" hidden="true">
       <c r="A87" t="s" s="2">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="B87" t="s" s="2">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="C87" s="2"/>
       <c r="D87" t="s" s="2">
@@ -14405,10 +14413,10 @@
         <v>181</v>
       </c>
       <c r="L87" t="s" s="2">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="M87" t="s" s="2">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="N87" s="2"/>
       <c r="O87" s="2"/>
@@ -14435,13 +14443,13 @@
         <v>88</v>
       </c>
       <c r="X87" t="s" s="2">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="Y87" t="s" s="2">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="Z87" t="s" s="2">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="AA87" t="s" s="2">
         <v>88</v>
@@ -14459,7 +14467,7 @@
         <v>88</v>
       </c>
       <c r="AF87" t="s" s="2">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="AG87" t="s" s="2">
         <v>86</v>
@@ -14504,7 +14512,7 @@
         <v>88</v>
       </c>
       <c r="AU87" t="s" s="2">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="AV87" t="s" s="2">
         <v>88</v>
@@ -14515,10 +14523,10 @@
     </row>
     <row r="88" hidden="true">
       <c r="A88" t="s" s="2">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="B88" t="s" s="2">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="C88" s="2"/>
       <c r="D88" t="s" s="2">
@@ -14541,13 +14549,13 @@
         <v>88</v>
       </c>
       <c r="K88" t="s" s="2">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="L88" t="s" s="2">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="M88" t="s" s="2">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="N88" s="2"/>
       <c r="O88" s="2"/>
@@ -14598,7 +14606,7 @@
         <v>88</v>
       </c>
       <c r="AF88" t="s" s="2">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="AG88" t="s" s="2">
         <v>86</v>
@@ -14643,21 +14651,21 @@
         <v>88</v>
       </c>
       <c r="AU88" t="s" s="2">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="AV88" t="s" s="2">
         <v>88</v>
       </c>
       <c r="AW88" t="s" s="2">
-        <v>567</v>
+        <v>568</v>
       </c>
     </row>
     <row r="89" hidden="true">
       <c r="A89" t="s" s="2">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="B89" t="s" s="2">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="C89" s="2"/>
       <c r="D89" t="s" s="2">
@@ -14680,13 +14688,13 @@
         <v>88</v>
       </c>
       <c r="K89" t="s" s="2">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="L89" t="s" s="2">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="M89" t="s" s="2">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="N89" s="2"/>
       <c r="O89" s="2"/>
@@ -14737,7 +14745,7 @@
         <v>88</v>
       </c>
       <c r="AF89" t="s" s="2">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="AG89" t="s" s="2">
         <v>86</v>
@@ -14749,7 +14757,7 @@
         <v>88</v>
       </c>
       <c r="AJ89" t="s" s="2">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="AK89" t="s" s="2">
         <v>88</v>
@@ -14782,7 +14790,7 @@
         <v>88</v>
       </c>
       <c r="AU89" t="s" s="2">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="AV89" t="s" s="2">
         <v>88</v>
@@ -14793,10 +14801,10 @@
     </row>
     <row r="90" hidden="true">
       <c r="A90" t="s" s="2">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="B90" t="s" s="2">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="C90" s="2"/>
       <c r="D90" t="s" s="2">
@@ -14932,10 +14940,10 @@
     </row>
     <row r="91" hidden="true">
       <c r="A91" t="s" s="2">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="B91" t="s" s="2">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="C91" s="2"/>
       <c r="D91" t="s" s="2">
@@ -15073,14 +15081,14 @@
     </row>
     <row r="92" hidden="true">
       <c r="A92" t="s" s="2">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="B92" t="s" s="2">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="C92" s="2"/>
       <c r="D92" t="s" s="2">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="E92" s="2"/>
       <c r="F92" t="s" s="2">
@@ -15102,10 +15110,10 @@
         <v>141</v>
       </c>
       <c r="L92" t="s" s="2">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="M92" t="s" s="2">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="N92" t="s" s="2">
         <v>167</v>
@@ -15158,7 +15166,7 @@
         <v>88</v>
       </c>
       <c r="AF92" t="s" s="2">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="AG92" t="s" s="2">
         <v>86</v>
@@ -15214,10 +15222,10 @@
     </row>
     <row r="93" hidden="true">
       <c r="A93" t="s" s="2">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="B93" t="s" s="2">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="C93" s="2"/>
       <c r="D93" t="s" s="2">
@@ -15243,10 +15251,10 @@
         <v>181</v>
       </c>
       <c r="L93" t="s" s="2">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="M93" t="s" s="2">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="N93" s="2"/>
       <c r="O93" s="2"/>
@@ -15273,13 +15281,13 @@
         <v>88</v>
       </c>
       <c r="X93" t="s" s="2">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="Y93" t="s" s="2">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="Z93" t="s" s="2">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="AA93" t="s" s="2">
         <v>88</v>
@@ -15297,7 +15305,7 @@
         <v>88</v>
       </c>
       <c r="AF93" t="s" s="2">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="AG93" t="s" s="2">
         <v>86</v>
@@ -15342,7 +15350,7 @@
         <v>88</v>
       </c>
       <c r="AU93" t="s" s="2">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="AV93" t="s" s="2">
         <v>88</v>
@@ -15353,14 +15361,14 @@
     </row>
     <row r="94" hidden="true">
       <c r="A94" t="s" s="2">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="B94" t="s" s="2">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="C94" s="2"/>
       <c r="D94" t="s" s="2">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="E94" s="2"/>
       <c r="F94" t="s" s="2">
@@ -15379,13 +15387,13 @@
         <v>88</v>
       </c>
       <c r="K94" t="s" s="2">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="L94" t="s" s="2">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="M94" t="s" s="2">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="N94" s="2"/>
       <c r="O94" s="2"/>
@@ -15436,7 +15444,7 @@
         <v>88</v>
       </c>
       <c r="AF94" t="s" s="2">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="AG94" t="s" s="2">
         <v>96</v>
@@ -15451,7 +15459,7 @@
         <v>88</v>
       </c>
       <c r="AK94" t="s" s="2">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="AL94" t="s" s="2">
         <v>88</v>
@@ -15463,7 +15471,7 @@
         <v>88</v>
       </c>
       <c r="AO94" t="s" s="2">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="AP94" t="s" s="2">
         <v>88</v>
@@ -15472,7 +15480,7 @@
         <v>88</v>
       </c>
       <c r="AR94" t="s" s="2">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="AS94" t="s" s="2">
         <v>88</v>
@@ -15481,7 +15489,7 @@
         <v>88</v>
       </c>
       <c r="AU94" t="s" s="2">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="AV94" t="s" s="2">
         <v>88</v>
@@ -15492,10 +15500,10 @@
     </row>
     <row r="95" hidden="true">
       <c r="A95" t="s" s="2">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="B95" t="s" s="2">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="C95" s="2"/>
       <c r="D95" t="s" s="2">
@@ -15518,19 +15526,19 @@
         <v>88</v>
       </c>
       <c r="K95" t="s" s="2">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="L95" t="s" s="2">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="M95" t="s" s="2">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="N95" t="s" s="2">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="O95" t="s" s="2">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="P95" t="s" s="2">
         <v>88</v>
@@ -15579,7 +15587,7 @@
         <v>88</v>
       </c>
       <c r="AF95" t="s" s="2">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="AG95" t="s" s="2">
         <v>86</v>
@@ -15624,7 +15632,7 @@
         <v>88</v>
       </c>
       <c r="AU95" t="s" s="2">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="AV95" t="s" s="2">
         <v>88</v>
@@ -15635,10 +15643,10 @@
     </row>
     <row r="96" hidden="true">
       <c r="A96" t="s" s="2">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="B96" t="s" s="2">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="C96" s="2"/>
       <c r="D96" t="s" s="2">
@@ -15664,13 +15672,13 @@
         <v>181</v>
       </c>
       <c r="L96" t="s" s="2">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="M96" t="s" s="2">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="N96" t="s" s="2">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="O96" s="2"/>
       <c r="P96" t="s" s="2">
@@ -15696,13 +15704,13 @@
         <v>88</v>
       </c>
       <c r="X96" t="s" s="2">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="Y96" t="s" s="2">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="Z96" t="s" s="2">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="AA96" t="s" s="2">
         <v>88</v>
@@ -15720,7 +15728,7 @@
         <v>88</v>
       </c>
       <c r="AF96" t="s" s="2">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="AG96" t="s" s="2">
         <v>86</v>
@@ -15765,7 +15773,7 @@
         <v>88</v>
       </c>
       <c r="AU96" t="s" s="2">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="AV96" t="s" s="2">
         <v>88</v>

</xml_diff>